<commit_message>
Finalize D5 publication validation and audits
</commit_message>
<xml_diff>
--- a/Project 1 Data Quality Assessment/D5 Topological Role Consistency and Structural Representativeness/outputs/local/D5_audit_log.xlsx
+++ b/Project 1 Data Quality Assessment/D5 Topological Role Consistency and Structural Representativeness/outputs/local/D5_audit_log.xlsx
@@ -1104,7 +1104,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C93"/>
+  <dimension ref="A1:C123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1131,11 +1131,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>19291</v>
+        <v>24952</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>d289f2ed1790125576e6208aa59e739e900544fd5a3d6de3b66e4b01af1ed4ec</t>
+          <t>fc561940849ad26d15c8d38f28c15b2a69532720e790e08caf8cefe4150a7a2f</t>
         </is>
       </c>
     </row>
@@ -1146,11 +1146,11 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2837</v>
+        <v>3875</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>c2abac4e644f6aa39140b77b7df71f2d5841d4f280544fedb43d94acbe3d2b0d</t>
+          <t>4efe7ee048fe969fcb278e5ff2d86af60c91b20739989b3115d0903fc23cf4b6</t>
         </is>
       </c>
     </row>
@@ -1457,1048 +1457,1498 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>outputs/figures/figure_bundle_audit.json</t>
+          <t>outputs/figures/FigD5_6_validation_coverage.pdf</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>2409</v>
+        <v>55784</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>da3ebd141c082e91a1745abc60394a9bc5c09de0cd31ad6297aa5cafc4d49756</t>
+          <t>bcb82f3433cc8c9bff8b96a4bdab30af87da622e94f7769341fb0cbb80a699ab</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>outputs/local/D5_ablation_redundancy.xlsx</t>
+          <t>outputs/figures/FigD5_6_validation_coverage.png</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>9987</v>
+        <v>638508</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>78516d5fee705aee9308c5ece95ce07cb2b09aec93248e68b486446b52ecd559</t>
+          <t>0e727c79d832125c2692a90737a1549169a2e462708c6e7ca453c71ee724c956</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>outputs/local/D5_admission_decision.json</t>
+          <t>outputs/figures/FigD5_6_validation_coverage.svg</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>588</v>
+        <v>69107</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>a9c40d2d57897245afa23202d8e7ba49245ff63b19b9427ab86d12003a4c1583</t>
+          <t>924185eb051252194293bb1f0f626a326a8fbab06ed4f94bd5482f9f20ba171d</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>outputs/local/D5_admission_decision.xlsx</t>
+          <t>outputs/figures/FigD5_6_validation_coverage.tiff</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>6135</v>
+        <v>1372644</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>96cce073f38f1f8e9d436722f18513ea84f6acf4ba33920ca07d1185db5767dd</t>
+          <t>eda63abf34b431710ff6444936d9b430fec8c42fc9b6c0e4b0053d7a93527571</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>outputs/local/D5_audit_log.xlsx</t>
+          <t>outputs/figures/FigD5_7_D4_D5_complementarity.pdf</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>72619</v>
+        <v>56584</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>cea6bec15bebf22e5b642e374362165e070b1a825e2c905d22c5885728698aa8</t>
+          <t>34558954fd2e7ff1dde3e9533847ae7334f7f41df775b4848784826ec78afc9b</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>outputs/local/D5_case_study_exports.xlsx</t>
+          <t>outputs/figures/FigD5_7_D4_D5_complementarity.png</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>44198</v>
+        <v>570614</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>060027cb3475620e45c16a5aed24ec4f94b00c01a7a3ba027a188963d7682dbc</t>
+          <t>c841a08eced4705db43bea80ef95f51318deed8cbc9fa59162af958206f7ec14</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>outputs/local/D5_edge_profile_summary.xlsx</t>
+          <t>outputs/figures/FigD5_7_D4_D5_complementarity.svg</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>26857</v>
+        <v>53698</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>5b3bd2c7f60bb706732433cc146f79297976ea8f202150b40c281c932b3a6329</t>
+          <t>d2a60d2df159dd5773262648198d95fa05aa2dfc6b36ea5ca4208c6b7b421ed5</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>outputs/local/D5_event_windows.parquet</t>
+          <t>outputs/figures/FigD5_7_D4_D5_complementarity.tiff</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>80614</v>
+        <v>1364872</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2874ab1d42be1723d6baabd3bd81b768d9f4b3fcf5459712e226f029f25a24fd</t>
+          <t>deff101f038b17d4bd5a4545fd371aa0c588c56565c5238d555bfb4471899aa1</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>outputs/local/D5_event_windows.xlsx</t>
+          <t>outputs/figures/figure_bundle_audit.json</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>140097</v>
+        <v>2409</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>97f101d88e4b67e9376735a772083ed8f1403eb700de6666b4a51314b7bc3dae</t>
+          <t>da3ebd141c082e91a1745abc60394a9bc5c09de0cd31ad6297aa5cafc4d49756</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>outputs/local/D5_gate_interface.parquet</t>
+          <t>outputs/local/D5_ablation_redundancy.xlsx</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>796803</v>
+        <v>9984</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>22b640fa64ff95f0677bdcafea1517c192dd506fc11559efc53db49916918e0e</t>
+          <t>f0feb1f3c9868bf39b167645436a3c13adea0cb6253ce840188905750b8c2157</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>outputs/local/D5_gate_interface.schema.json</t>
+          <t>outputs/local/D5_admission_decision.json</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>1106</v>
+        <v>588</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>215cbcde37b7836586e81e198c982e82561c42170ddda3ef2bf109052fb10e29</t>
+          <t>a9c40d2d57897245afa23202d8e7ba49245ff63b19b9427ab86d12003a4c1583</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>outputs/local/D5_gate_interface.xlsx</t>
+          <t>outputs/local/D5_admission_decision.xlsx</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>5209423</v>
+        <v>6135</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>cc6458fcb96aa750a01b53bb7acfaceae4f832b53e68bd1840f57a8ee787b22c</t>
+          <t>96cce073f38f1f8e9d436722f18513ea84f6acf4ba33920ca07d1185db5767dd</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>outputs/local/D5_main_scores_hourly.parquet</t>
+          <t>outputs/local/D5_audit_log.xlsx</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>7340495</v>
+        <v>74702</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>64274562d7139d510dd3780dbd67bd2c2c5913908dbbec8ac7d4bcceb0418cd1</t>
+          <t>675cf312d5aa5e97cb8f722b22af3a9782c2b91a9dd3f12f708cfd6bb4955e3c</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>outputs/local/D5_main_scores_hourly.xlsx</t>
+          <t>outputs/local/D5_case_study_exports.xlsx</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>45272583</v>
+        <v>44198</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2ae0e3dcb195bddabcb98ac87479345348da28818c565a978c56f75ff0ee19c9</t>
+          <t>060027cb3475620e45c16a5aed24ec4f94b00c01a7a3ba027a188963d7682dbc</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>outputs/local/D5_mapping_params.xlsx</t>
+          <t>outputs/local/D5_edge_profile_summary.xlsx</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>20237</v>
+        <v>26857</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>30ffe256d465c57c614fcab9fa40d92fcd68a7c1f5fc78cbd8e0e0d00779b6a6</t>
+          <t>5b3bd2c7f60bb706732433cc146f79297976ea8f202150b40c281c932b3a6329</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>outputs/local/D5_multiscale_aggregates.xlsx</t>
+          <t>outputs/local/D5_event_windows.parquet</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>1060062</v>
+        <v>80614</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>96da07e011eecb169c1880e11e5c8656c9aa16a62434b3ad540a8b9a658a5da0</t>
+          <t>2874ab1d42be1723d6baabd3bd81b768d9f4b3fcf5459712e226f029f25a24fd</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>outputs/local/D5_reference_window_library.parquet</t>
+          <t>outputs/local/D5_event_windows.xlsx</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>62947</v>
+        <v>140097</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>b84bd8208e2e533e83c722868f022eaf87e07991f184e6d59e9411909e5360bc</t>
+          <t>97f101d88e4b67e9376735a772083ed8f1403eb700de6666b4a51314b7bc3dae</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>outputs/local/D5_reference_window_library.xlsx</t>
+          <t>outputs/local/D5_gate_interface.parquet</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>228952</v>
+        <v>796803</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>12bb084003accca5fd0e85f42191286a56a27c7016b617296cde45ff4004edf1</t>
+          <t>22b640fa64ff95f0677bdcafea1517c192dd506fc11559efc53db49916918e0e</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>outputs/local/D5_regime_state.parquet</t>
+          <t>outputs/local/D5_gate_interface.schema.json</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>3658910</v>
+        <v>1128</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>622dd0f5ed1473ae5de464e4207e51ff9470de209cadcee9b30cbac92f9392e8</t>
+          <t>619b0d9ef22475a5de39a752b479540987d05f9cb5d649e2f7bece38005622f3</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>outputs/local/D5_regime_state.xlsx</t>
+          <t>outputs/local/D5_gate_interface.xlsx</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>45834835</v>
+        <v>5209423</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>427fe81df8b7861210e267f694058376a754fa724e0bbafe1b07208e32787485</t>
+          <t>cc6458fcb96aa750a01b53bb7acfaceae4f832b53e68bd1840f57a8ee787b22c</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>outputs/local/D5_report_interface.parquet</t>
+          <t>outputs/local/D5_main_scores_hourly.parquet</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>1171194</v>
+        <v>7340495</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>f057e0a8037282fb43a71a94d7043c7bd3de2b4c8fa9865365bcf0427195dbda</t>
+          <t>64274562d7139d510dd3780dbd67bd2c2c5913908dbbec8ac7d4bcceb0418cd1</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>outputs/local/D5_report_interface.schema.json</t>
+          <t>outputs/local/D5_main_scores_hourly.xlsx</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>834</v>
+        <v>45272583</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>e697ed5d3e9ba3b4ae628350d5592c7c5932a3326ac3721df45953d8e3569c87</t>
+          <t>2ae0e3dcb195bddabcb98ac87479345348da28818c565a978c56f75ff0ee19c9</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>outputs/local/D5_report_interface.xlsx</t>
+          <t>outputs/local/D5_mapping_params.xlsx</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>11410677</v>
+        <v>20237</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>f9040450b3fb8204f2fea44f92c003d1cdc2acf900a29715ee732a8b9b450aae</t>
+          <t>30ffe256d465c57c614fcab9fa40d92fcd68a7c1f5fc78cbd8e0e0d00779b6a6</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>outputs/local/D5_sensor_influence.parquet</t>
+          <t>outputs/local/D5_multiscale_aggregates.xlsx</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>6011187</v>
+        <v>1060062</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>a9270494760fcb4ae501abcf54c50e813ca74d6306d7fbca94d7ef1a1d1730a2</t>
+          <t>96da07e011eecb169c1880e11e5c8656c9aa16a62434b3ad540a8b9a658a5da0</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>outputs/local/D5_sensor_influence.xlsx</t>
+          <t>outputs/local/D5_reference_window_library.parquet</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>16403976</v>
+        <v>62947</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>338920c1db9c7b1bc500fa43d92f02f6165187545a79f696771287bfd877a9a0</t>
+          <t>b84bd8208e2e533e83c722868f022eaf87e07991f184e6d59e9411909e5360bc</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>outputs/local/D5_sensor_profile_summary.xlsx</t>
+          <t>outputs/local/D5_reference_window_library.xlsx</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>7442</v>
+        <v>228952</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>aef38bd66378a9ae3b2c76a848f1ef4d51d504616c435440e45f99eadf9fb5a9</t>
+          <t>12bb084003accca5fd0e85f42191286a56a27c7016b617296cde45ff4004edf1</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>outputs/local/D5_spatial_evidence.parquet</t>
+          <t>outputs/local/D5_regime_state.parquet</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>6146048</v>
+        <v>3658910</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>4edb2bd1af0cbdac8fc61382508099137349f67f6ce70da4ee1831848bfe3733</t>
+          <t>622dd0f5ed1473ae5de464e4207e51ff9470de209cadcee9b30cbac92f9392e8</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>outputs/local/D5_spatial_evidence.xlsx</t>
+          <t>outputs/local/D5_regime_state.xlsx</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>15958642</v>
+        <v>45834835</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>6e2a433bcdb115b841f269c5eb5184623502c7221234da51b8ade0377c120327</t>
+          <t>427fe81df8b7861210e267f694058376a754fa724e0bbafe1b07208e32787485</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>outputs/local/D5_spatial_templates.template_bundle.json</t>
+          <t>outputs/local/D5_report_interface.parquet</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>542571</v>
+        <v>1171194</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>704238fcb5551593e569bdb3e015f04cb710815fdeccbb8aa28ba9a0c7e59ace</t>
+          <t>f057e0a8037282fb43a71a94d7043c7bd3de2b4c8fa9865365bcf0427195dbda</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>outputs/local/D5_spatial_templates.xlsx</t>
+          <t>outputs/local/D5_report_interface.schema.json</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>190694</v>
+        <v>853</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>6fc3291e19dd0663ccd33db897edbf39e67f54e7db7b1fa8de0648d06d82c6bc</t>
+          <t>c740ff5a12c99a1a761c5f2ab45d12f5174aaac3b2201e58e6d67a1a8c87c06e</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>outputs/local/D5_support_assessment.parquet</t>
+          <t>outputs/local/D5_report_interface.xlsx</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>52815</v>
+        <v>11410677</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>00d3ed69dc3899db48c841bb56c6664bc1832e365fd5fa5c13130b6d231e5750</t>
+          <t>f9040450b3fb8204f2fea44f92c003d1cdc2acf900a29715ee732a8b9b450aae</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>outputs/local/D5_support_assessment.xlsx</t>
+          <t>outputs/local/D5_sensor_influence.parquet</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>28036</v>
+        <v>6011187</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>34df65d8e4329d166c69a9bc505bb97a8397e537f323c5be392fba093827dd98</t>
+          <t>a9270494760fcb4ae501abcf54c50e813ca74d6306d7fbca94d7ef1a1d1730a2</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>outputs/local/D5_topology_drift_alerts.parquet</t>
+          <t>outputs/local/D5_sensor_influence.xlsx</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>10824</v>
+        <v>16403976</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>59d05a6c138fc18e295611bb0e39f469c07f6a25522ed809ea4f76ca018a908a</t>
+          <t>338920c1db9c7b1bc500fa43d92f02f6165187545a79f696771287bfd877a9a0</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>outputs/local/D5_topology_drift_alerts.xlsx</t>
+          <t>outputs/local/D5_sensor_profile_summary.xlsx</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>9965</v>
+        <v>7442</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>7262caaddcf1713a512e6dd52157f3f0e4bee9ae2642dcaf63eed60ff9ce9a87</t>
+          <t>aef38bd66378a9ae3b2c76a848f1ef4d51d504616c435440e45f99eadf9fb5a9</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>outputs/local/D5_topology_evidence.yaml</t>
+          <t>outputs/local/D5_spatial_evidence.parquet</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>2342</v>
+        <v>6146048</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>50abd276a9e6bbf26acb9a22d3a796ca63423d363a036422dc57c6bdfeb71920</t>
+          <t>4edb2bd1af0cbdac8fc61382508099137349f67f6ce70da4ee1831848bfe3733</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>outputs/local/D5_topology_registry.json</t>
+          <t>outputs/local/D5_spatial_evidence.xlsx</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>14821</v>
+        <v>15958642</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>6efbf6722e2caecabf2d9999637d48bbb7c4d630dc3e9354982ed89d750965bc</t>
+          <t>6e2a433bcdb115b841f269c5eb5184623502c7221234da51b8ade0377c120327</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>outputs/local/D5_topology_registry.schema.json</t>
+          <t>outputs/local/D5_spatial_templates.template_bundle.json</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>1263</v>
+        <v>542571</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>3b6af16c6f624602a9851d780a2eb0d87f381ca851177c422c742d7fb60aed41</t>
+          <t>704238fcb5551593e569bdb3e015f04cb710815fdeccbb8aa28ba9a0c7e59ace</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>outputs/local/D5_topology_registry.xlsx</t>
+          <t>outputs/local/D5_spatial_templates.xlsx</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>11679</v>
+        <v>190694</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>7aa5db4087c2346acc99d827f7c3a0bd49ce90540fb2ec8f56664c82b14e36ff</t>
+          <t>6fc3291e19dd0663ccd33db897edbf39e67f54e7db7b1fa8de0648d06d82c6bc</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>outputs/local/D5_topology_registry.yaml</t>
+          <t>outputs/local/D5_support_assessment.parquet</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>2838</v>
+        <v>52815</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>46e191549a0c768ee947bff4d98f26f38a93ecbce380ab4ff8114d2885dd29f9</t>
+          <t>00d3ed69dc3899db48c841bb56c6664bc1832e365fd5fa5c13130b6d231e5750</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>outputs/local/D5_validation_results.xlsx</t>
+          <t>outputs/local/D5_support_assessment.xlsx</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>60790</v>
+        <v>28036</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>3eff800b27bf69ec156f8138888d8c70af6d283d82e144d64162ae3ad416b651</t>
+          <t>34df65d8e4329d166c69a9bc505bb97a8397e537f323c5be392fba093827dd98</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>outputs/local/D5_zone_consensus.parquet</t>
+          <t>outputs/local/D5_topology_drift_alerts.parquet</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>1618880</v>
+        <v>10824</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>0cb43651f4dc8c4a7f378cfe3be964a688e7df7a2ff45052f649259b415cdb8c</t>
+          <t>59d05a6c138fc18e295611bb0e39f469c07f6a25522ed809ea4f76ca018a908a</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>outputs/local/D5_zone_consensus.xlsx</t>
+          <t>outputs/local/D5_topology_drift_alerts.xlsx</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>7277838</v>
+        <v>9965</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>f43c5554c5a0c9f3e50e38f51bc0db270a9c819c3a00a9f3dc23ae658b7e7149</t>
+          <t>7262caaddcf1713a512e6dd52157f3f0e4bee9ae2642dcaf63eed60ff9ce9a87</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>outputs/plot_data/D5_plot_data.csv</t>
+          <t>outputs/local/D5_topology_evidence.yaml</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>18506701</v>
+        <v>2342</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>f074d7394f60df5f9b874734fe644757863bf44e876dd97303344227afe065c3</t>
+          <t>50abd276a9e6bbf26acb9a22d3a796ca63423d363a036422dc57c6bdfeb71920</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>outputs/plot_data/D5_plot_data.parquet</t>
+          <t>outputs/local/D5_topology_registry.json</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>744459</v>
+        <v>14821</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>3236229f520cfa38329877aa013a7233229a77567e32c95b37a87d5fe94a5dd8</t>
+          <t>6efbf6722e2caecabf2d9999637d48bbb7c4d630dc3e9354982ed89d750965bc</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>outputs/plot_data/D5_plot_data_manifest.json</t>
+          <t>outputs/local/D5_topology_registry.schema.json</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>519</v>
+        <v>1301</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>27ae5a05d462aab27e6a6359daaf99d931840e8b58d462da108ff3ca12dfc1ae</t>
+          <t>0f4c6e9e6d510996d1435efd1810b4a1eaca35a989b7f3d78187e29f8ce9584e</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_CURRENT_RELEASE.md</t>
+          <t>outputs/local/D5_topology_registry.xlsx</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>837</v>
+        <v>11679</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>f627a6c9567b234ae0b9c61c2b0681a6c7a74f46d30cb9f48806c4fa7e7ca7ed</t>
+          <t>7aa5db4087c2346acc99d827f7c3a0bd49ce90540fb2ec8f56664c82b14e36ff</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_EXPERT_REPORT_v2.1.docx</t>
+          <t>outputs/local/D5_topology_registry.yaml</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>2047657</v>
+        <v>2838</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>8e5db363b70bd05b8584eb191b764d1d2beee31c2be738b56f44c9902c67fb04</t>
+          <t>46e191549a0c768ee947bff4d98f26f38a93ecbce380ab4ff8114d2885dd29f9</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_EXPERT_REPORT_v2.1.md</t>
+          <t>outputs/local/D5_validation_results.xlsx</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>7814</v>
+        <v>64326</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>6de0e55c9c7f57f2c030d48076b3da316a94d53167e1c1e9d164031972691657</t>
+          <t>b4a0f5586b1108b945dba84b87a47a7f387c11fa182de0c506977f3c9870efff</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_EXPERT_REPORT_v2.2.docx</t>
+          <t>outputs/local/D5_zone_consensus.parquet</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>2107226</v>
+        <v>1618880</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>9dfbe96a145765a0e22e8452ec1a76f759ae52cd201b71694aa7c7e815fd8d8b</t>
+          <t>0cb43651f4dc8c4a7f378cfe3be964a688e7df7a2ff45052f649259b415cdb8c</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_EXPERT_REPORT_v2.2.md</t>
+          <t>outputs/local/D5_zone_consensus.xlsx</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>8480</v>
+        <v>7277838</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>5f9333b22a9d8dc1b40d9ac2f1f684ee851785bf1f742be406e6433cfc841cfd</t>
+          <t>f43c5554c5a0c9f3e50e38f51bc0db270a9c819c3a00a9f3dc23ae658b7e7149</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_EXPERT_REPORT_v2.3.docx</t>
+          <t>outputs/plot_data/D5_plot_data.csv</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>2056532</v>
+        <v>18506701</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>19b15492f9b09b02820cf4ff0effd41c672a7dd0a99a42eef3886c732b622fe5</t>
+          <t>f074d7394f60df5f9b874734fe644757863bf44e876dd97303344227afe065c3</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_EXPERT_REPORT_v2.3.md</t>
+          <t>outputs/plot_data/D5_plot_data.parquet</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>9043</v>
+        <v>744459</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>93baa7ffe8d1d92abac60ce6896dd742d71410bb89c771ab5d8e73c9bc3d6b57</t>
+          <t>3236229f520cfa38329877aa013a7233229a77567e32c95b37a87d5fe94a5dd8</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_FIGURE_CAPTIONS_v2.1.md</t>
+          <t>outputs/plot_data/D5_plot_data_manifest.json</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>2282</v>
+        <v>519</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>dd5ca9eea1365f682a5166e6f8e11da3da1b6ce06652795ba6bd0112a5711bc0</t>
+          <t>27ae5a05d462aab27e6a6359daaf99d931840e8b58d462da108ff3ca12dfc1ae</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_FIGURE_CAPTIONS_v2.2.md</t>
+          <t>outputs/publication/D5_coverage_strata.parquet</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>2185</v>
+        <v>5837</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>4e3e50df15c243b7c789337fb51e9fe8f350c3815f05b408b6dd2f8aad9c4067</t>
+          <t>f4da589996c29b4e710131be262c3efdaa0fb822e051293f1310365aaf0e7b75</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_FIGURE_CAPTIONS_v2.3.md</t>
+          <t>outputs/publication/D5_coverage_summary.parquet</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>2471</v>
+        <v>2879</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>5aace3b407bf260ee6a54a95a25736b01d1ec2831a95823a45288d40270b532c</t>
+          <t>54201e6be7009f8ed97eb53e8abd9d8d33766757486839e1d1650d09bf1718c6</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_PROJECT_DIRECTORY_GUIDE_v2.1.docx</t>
+          <t>outputs/publication/D5_d4_d5_composite.parquet</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>40336</v>
+        <v>4352</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>c2da3e9cca5ef0a5e83b63089e8deeb7299a7e0e7735c0b4751cd47f2fc47844</t>
+          <t>54eed66c77212702829f3d4bc85907babd66e415997082a0a86a8b49ea1b4556</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_PROJECT_DIRECTORY_GUIDE_v2.1.md</t>
+          <t>outputs/publication/D5_d4_d5_dependence.parquet</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>5333</v>
+        <v>4364</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>0303a5bbdc16689493eb5b3826d95bf7c23fc4405284ef7db01d13b5a1d1b045</t>
+          <t>a18b2d57e0affd0fdf036d32f43b988f92c6866b4300aa8cfa798991759f1268</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_PROJECT_DIRECTORY_GUIDE_v2.2.docx</t>
+          <t>outputs/publication/D5_decision_register.parquet</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>40363</v>
+        <v>4691</v>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>eada32c51f435a6355dc873b748b4f894cbbc17bedfc4be6090371aa323aea5e</t>
+          <t>8c888a1b2a0a3790d1333395853deb23b7c145c3a9489c8464c595fef28427f9</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_PROJECT_DIRECTORY_GUIDE_v2.2.md</t>
+          <t>outputs/publication/D5_localization.parquet</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>5307</v>
+        <v>6980</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>b63d3b48b8902ad31fcbeac70f218c2c3abd2b1ee4293aff45cbc89fe16b950b</t>
+          <t>e63682e2c8a0ebeb772d9d0eae21b4be654b370f853eb939376249c595ddfcff</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_PROJECT_DIRECTORY_GUIDE_v2.3.docx</t>
+          <t>outputs/publication/D5_monthly_coverage.parquet</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>40364</v>
+        <v>6919</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>788d71134331e7d994e157cbfb511ef1f5966eb546d05ea3a77a8b2dd90c2fce</t>
+          <t>51e4fd571650b85d5e4d8c2aab7c0ca543cb81aff01517a7efacc70c08bea506</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_PROJECT_DIRECTORY_GUIDE_v2.3.md</t>
+          <t>outputs/publication/D5_outer_refit_deltas.parquet</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>5459</v>
+        <v>7921</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>0308ed8c677cbbb3581e4022bbc99623af3de79cf83fc9283b160fd54cb8d503</t>
+          <t>1601955bc59dfd0da87cd33e695f16ac974ad0be8ecacbdb23dfe465599ce7bf</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>outputs/reports/nature_figure_bundle_audit.json</t>
+          <t>outputs/publication/D5_outer_refit_summary.parquet</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>2409</v>
+        <v>6681</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>da3ebd141c082e91a1745abc60394a9bc5c09de0cd31ad6297aa5cafc4d49756</t>
+          <t>9ea7de7e9e34e2bc3b5c657dd72bded594918e0310ad7e231a2610ef45253f30</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>outputs/sensitivity/D5_sensitivity_manifest.json</t>
+          <t>outputs/publication/D5_publication_audit_manifest.json</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>2345</v>
+        <v>4364</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>71ddb925f1c43c2bb363be78cb221f6a90ed9d1bce2beb713989957efcb0b8d8</t>
+          <t>e3fb4bafbf07c9310f2c5afae1737d00b609f7d8c0f563b1d51366aab2cd3df3</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>outputs/sensitivity/D5_shadow_scores.parquet</t>
+          <t>outputs/publication/D5_publication_audit_tables.xlsx</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>2987712</v>
+        <v>23665</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>a54b95d4cada7ab1f9a1e4bd7723d29f46c9e3c19de2bcab6f52a9da161ba5fc</t>
+          <t>f804b0704ef36c432f26f3faf80d6ad7cbf93f014ec02a34916644a509ae3dae</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>outputs/sensitivity/D5_shadow_scores.xlsx</t>
+          <t>outputs/publication/D5_PUBLICATION_READINESS_AUDIT_v1.0.md</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>10004039</v>
+        <v>5709</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>1229f93be5258226bfbdc36daab2ceb3aa2b475485c1fa0392cc15ec148a97f9</t>
+          <t>951b14afceb659a941306c90c0763fec61bf79de8cd0d5316024059cfbdf7bdf</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>outputs/sensitivity/D5_shadow_template_shift.xlsx</t>
+          <t>outputs/publication/D5_risk_coverage.parquet</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>41680</v>
+        <v>5064</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>3f68e2e6f4d6bc46aa021613f6b8ee25bb562d0798f1896ef47555b36c89fe35</t>
+          <t>eb0caf68ddfdc8203a64254c3aa277304432bb3fa762cb19e0b9123740a49508</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>outputs/sensitivity/D5_track_invariance.xlsx</t>
+          <t>outputs/publication/D5_support_sensitivity.parquet</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>14538</v>
+        <v>5871</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>c9ed72b9a91d1fa854692c1cabf77687a652bf9723a7d405b4fbc08cf5b6c1c0</t>
+          <t>f6ee73f3893ed53682e63122e9220948cc97ffa0c9ead47b20b6b2c739de9fda</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>outputs/shadow_v2/D5_graph_structure_learning_shadow.parquet</t>
+          <t>outputs/publication/D5_target_influence.parquet</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>9388</v>
+        <v>8536</v>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>f65546587bfb8c5a13efa5af7a38f57820bb3467cbd974c3bfad3c369a88f2c7</t>
+          <t>77b6a0a69423e32f3f664790ccd0b4e841d967fce6370559b159ea50c758bdad</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>outputs/shadow_v2/D5_graph_structure_learning_shadow.xlsx</t>
+          <t>outputs/publication/FigD5_6_validation_coverage_source_data.xlsx</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>8325</v>
+        <v>10606</v>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>b5a4109a1f1e707a2bc54497df9a808bd01cf23a9094aed4a77ff885fef49653</t>
+          <t>12a62815cd1300db24c3c293d091547a95a521a3b965009db4e36ff41493ada4</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
+          <t>outputs/publication/FigD5_7_D4_D5_complementarity_source_data.xlsx</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>9134</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>325b0094eb3ea93567482e7648b5740f141441b830fd2e540c5805c3120d5d52</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>outputs/reports/D5_CURRENT_RELEASE.md</t>
+        </is>
+      </c>
+      <c r="B94" t="n">
+        <v>916</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>de2a0d79f1cc37684c35cae1e61858482c4476d9951c724a1c28dd40af6c44d1</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>outputs/reports/D5_EXPERT_REPORT_v2.1.docx</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>2047657</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>8e5db363b70bd05b8584eb191b764d1d2beee31c2be738b56f44c9902c67fb04</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>outputs/reports/D5_EXPERT_REPORT_v2.1.md</t>
+        </is>
+      </c>
+      <c r="B96" t="n">
+        <v>7814</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>6de0e55c9c7f57f2c030d48076b3da316a94d53167e1c1e9d164031972691657</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>outputs/reports/D5_EXPERT_REPORT_v2.2.docx</t>
+        </is>
+      </c>
+      <c r="B97" t="n">
+        <v>2107226</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>9dfbe96a145765a0e22e8452ec1a76f759ae52cd201b71694aa7c7e815fd8d8b</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>outputs/reports/D5_EXPERT_REPORT_v2.2.md</t>
+        </is>
+      </c>
+      <c r="B98" t="n">
+        <v>8480</v>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>5f9333b22a9d8dc1b40d9ac2f1f684ee851785bf1f742be406e6433cfc841cfd</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>outputs/reports/D5_EXPERT_REPORT_v2.3.docx</t>
+        </is>
+      </c>
+      <c r="B99" t="n">
+        <v>2056532</v>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>19b15492f9b09b02820cf4ff0effd41c672a7dd0a99a42eef3886c732b622fe5</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>outputs/reports/D5_EXPERT_REPORT_v2.3.md</t>
+        </is>
+      </c>
+      <c r="B100" t="n">
+        <v>9043</v>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>93baa7ffe8d1d92abac60ce6896dd742d71410bb89c771ab5d8e73c9bc3d6b57</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>outputs/reports/D5_EXPERT_REPORT_v2.4.docx</t>
+        </is>
+      </c>
+      <c r="B101" t="n">
+        <v>3111730</v>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>cc1e9c76ec52cffba4e49f71fddbcc746efd6c195e41cfda57373264bd57078b</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>outputs/reports/D5_EXPERT_REPORT_v2.4.md</t>
+        </is>
+      </c>
+      <c r="B102" t="n">
+        <v>9532</v>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>fc5b363eb632924c649f82b46c9848f77eff3e0f4a430ceedd119e5b7542426c</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>outputs/reports/D5_FIGURE_CAPTIONS_v2.1.md</t>
+        </is>
+      </c>
+      <c r="B103" t="n">
+        <v>2282</v>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>dd5ca9eea1365f682a5166e6f8e11da3da1b6ce06652795ba6bd0112a5711bc0</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>outputs/reports/D5_FIGURE_CAPTIONS_v2.2.md</t>
+        </is>
+      </c>
+      <c r="B104" t="n">
+        <v>2185</v>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>4e3e50df15c243b7c789337fb51e9fe8f350c3815f05b408b6dd2f8aad9c4067</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>outputs/reports/D5_FIGURE_CAPTIONS_v2.3.md</t>
+        </is>
+      </c>
+      <c r="B105" t="n">
+        <v>2471</v>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>5aace3b407bf260ee6a54a95a25736b01d1ec2831a95823a45288d40270b532c</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>outputs/reports/D5_FIGURE_CAPTIONS_v2.4.md</t>
+        </is>
+      </c>
+      <c r="B106" t="n">
+        <v>3600</v>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>555abddc4fd206f1d6afe947be1fad9f7557a5162e37116fa4537fd8fcc087bb</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>outputs/reports/D5_PROJECT_DIRECTORY_GUIDE_v2.1.docx</t>
+        </is>
+      </c>
+      <c r="B107" t="n">
+        <v>40336</v>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>c2da3e9cca5ef0a5e83b63089e8deeb7299a7e0e7735c0b4751cd47f2fc47844</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>outputs/reports/D5_PROJECT_DIRECTORY_GUIDE_v2.1.md</t>
+        </is>
+      </c>
+      <c r="B108" t="n">
+        <v>5333</v>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>0303a5bbdc16689493eb5b3826d95bf7c23fc4405284ef7db01d13b5a1d1b045</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>outputs/reports/D5_PROJECT_DIRECTORY_GUIDE_v2.2.docx</t>
+        </is>
+      </c>
+      <c r="B109" t="n">
+        <v>40363</v>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>eada32c51f435a6355dc873b748b4f894cbbc17bedfc4be6090371aa323aea5e</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>outputs/reports/D5_PROJECT_DIRECTORY_GUIDE_v2.2.md</t>
+        </is>
+      </c>
+      <c r="B110" t="n">
+        <v>5307</v>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>b63d3b48b8902ad31fcbeac70f218c2c3abd2b1ee4293aff45cbc89fe16b950b</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>outputs/reports/D5_PROJECT_DIRECTORY_GUIDE_v2.3.docx</t>
+        </is>
+      </c>
+      <c r="B111" t="n">
+        <v>40364</v>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>788d71134331e7d994e157cbfb511ef1f5966eb546d05ea3a77a8b2dd90c2fce</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>outputs/reports/D5_PROJECT_DIRECTORY_GUIDE_v2.3.md</t>
+        </is>
+      </c>
+      <c r="B112" t="n">
+        <v>5459</v>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>0308ed8c677cbbb3581e4022bbc99623af3de79cf83fc9283b160fd54cb8d503</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>outputs/reports/D5_PROJECT_DIRECTORY_GUIDE_v2.4.docx</t>
+        </is>
+      </c>
+      <c r="B113" t="n">
+        <v>40366</v>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>3306d9a6afcb510e296a5c9031cbe916a059fb0c52e6431ad4ac8d67bf146f58</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>outputs/reports/D5_PROJECT_DIRECTORY_GUIDE_v2.4.md</t>
+        </is>
+      </c>
+      <c r="B114" t="n">
+        <v>5670</v>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>f68468aa772b22e9fd44f55c62997fa53699339f963e6de09346c7a502fec34e</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>outputs/reports/nature_figure_bundle_audit.json</t>
+        </is>
+      </c>
+      <c r="B115" t="n">
+        <v>2409</v>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>da3ebd141c082e91a1745abc60394a9bc5c09de0cd31ad6297aa5cafc4d49756</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>outputs/sensitivity/D5_sensitivity_manifest.json</t>
+        </is>
+      </c>
+      <c r="B116" t="n">
+        <v>2345</v>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>71ddb925f1c43c2bb363be78cb221f6a90ed9d1bce2beb713989957efcb0b8d8</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>outputs/sensitivity/D5_shadow_scores.parquet</t>
+        </is>
+      </c>
+      <c r="B117" t="n">
+        <v>2987712</v>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>a54b95d4cada7ab1f9a1e4bd7723d29f46c9e3c19de2bcab6f52a9da161ba5fc</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>outputs/sensitivity/D5_shadow_scores.xlsx</t>
+        </is>
+      </c>
+      <c r="B118" t="n">
+        <v>10004039</v>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>1229f93be5258226bfbdc36daab2ceb3aa2b475485c1fa0392cc15ec148a97f9</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>outputs/sensitivity/D5_shadow_template_shift.xlsx</t>
+        </is>
+      </c>
+      <c r="B119" t="n">
+        <v>41680</v>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>3f68e2e6f4d6bc46aa021613f6b8ee25bb562d0798f1896ef47555b36c89fe35</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>outputs/sensitivity/D5_track_invariance.xlsx</t>
+        </is>
+      </c>
+      <c r="B120" t="n">
+        <v>14538</v>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>c9ed72b9a91d1fa854692c1cabf77687a652bf9723a7d405b4fbc08cf5b6c1c0</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>outputs/shadow_v2/D5_graph_structure_learning_shadow.parquet</t>
+        </is>
+      </c>
+      <c r="B121" t="n">
+        <v>9388</v>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>f65546587bfb8c5a13efa5af7a38f57820bb3467cbd974c3bfad3c369a88f2c7</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>outputs/shadow_v2/D5_graph_structure_learning_shadow.xlsx</t>
+        </is>
+      </c>
+      <c r="B122" t="n">
+        <v>8325</v>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>b5a4109a1f1e707a2bc54497df9a808bd01cf23a9094aed4a77ff885fef49653</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
           <t>outputs/shadow_v2/D5_shadow_v2_manifest.json</t>
         </is>
       </c>
-      <c r="B93" t="n">
+      <c r="B123" t="n">
         <v>263</v>
       </c>
-      <c r="C93" t="inlineStr">
+      <c r="C123" t="inlineStr">
         <is>
           <t>b031365e134ba1bfee32dd92c04e35cdff1e904f78937c214e008540551a11f3</t>
         </is>

</xml_diff>

<commit_message>
Harden D5 integration and coverage audits
</commit_message>
<xml_diff>
--- a/Project 1 Data Quality Assessment/D5 Topological Role Consistency and Structural Representativeness/outputs/local/D5_audit_log.xlsx
+++ b/Project 1 Data Quality Assessment/D5 Topological Role Consistency and Structural Representativeness/outputs/local/D5_audit_log.xlsx
@@ -538,7 +538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -750,6 +750,36 @@
       <c r="C14" t="inlineStr">
         <is>
           <t>SVG/PDF/600dpi PNG/TIFF and frozen plot data</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>publication_artifact_hash_integrity</t>
+        </is>
+      </c>
+      <c r="B15" t="b">
+        <v>1</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>publication tables, source data and figure bundle match manifest SHA-256</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>d4_publication_dependency_current</t>
+        </is>
+      </c>
+      <c r="B16" t="b">
+        <v>0</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>exact single D4 run/calibration and main-score SHA-256; status=stale_dependency_blocked</t>
         </is>
       </c>
     </row>
@@ -1104,7 +1134,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C123"/>
+  <dimension ref="A1:C135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1131,11 +1161,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>24952</v>
+        <v>28805</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>fc561940849ad26d15c8d38f28c15b2a69532720e790e08caf8cefe4150a7a2f</t>
+          <t>2996a12d5c57570b074196dd8036c29032857b9fde93df7aea352aa371992c38</t>
         </is>
       </c>
     </row>
@@ -1146,11 +1176,11 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3875</v>
+        <v>4935</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>4efe7ee048fe969fcb278e5ff2d86af60c91b20739989b3115d0903fc23cf4b6</t>
+          <t>cfc1b4c9f71d05af39a974ef9463f90f52066b9e042c8f67b0930bec652f478f</t>
         </is>
       </c>
     </row>
@@ -1461,11 +1491,11 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>55784</v>
+        <v>54719</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>bcb82f3433cc8c9bff8b96a4bdab30af87da622e94f7769341fb0cbb80a699ab</t>
+          <t>ff8beec018d4d331224ef2236e7fbe172b41f929f356e23c19359572ec4fb2e3</t>
         </is>
       </c>
     </row>
@@ -1476,11 +1506,11 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>638508</v>
+        <v>656187</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>0e727c79d832125c2692a90737a1549169a2e462708c6e7ca453c71ee724c956</t>
+          <t>a5d0f89175f27a60c6eeca284615c672b5fa47f41fbbecf3c25d67ee17718553</t>
         </is>
       </c>
     </row>
@@ -1491,11 +1521,11 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>69107</v>
+        <v>69085</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>924185eb051252194293bb1f0f626a326a8fbab06ed4f94bd5482f9f20ba171d</t>
+          <t>60ed8eabe554b2a7c014a37929d2a8c0a6cf9253c107e31f49657ac47e37352b</t>
         </is>
       </c>
     </row>
@@ -1506,11 +1536,11 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>1372644</v>
+        <v>1389316</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>eda63abf34b431710ff6444936d9b430fec8c42fc9b6c0e4b0053d7a93527571</t>
+          <t>767b8e085c5fa28f4211ab49ed95097a666f52963742ae45fec71e2bfe93b160</t>
         </is>
       </c>
     </row>
@@ -1521,11 +1551,11 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>56584</v>
+        <v>58126</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>34558954fd2e7ff1dde3e9533847ae7334f7f41df775b4848784826ec78afc9b</t>
+          <t>1fc0731d8363ad2cc56a344a8b3410c920a9f51d34c938199548bfd4ef4d10a3</t>
         </is>
       </c>
     </row>
@@ -1536,11 +1566,11 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>570614</v>
+        <v>556320</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>c841a08eced4705db43bea80ef95f51318deed8cbc9fa59162af958206f7ec14</t>
+          <t>f4ee30551e441baa0c19c936f58a704a215e523c88e99bdec6a4f281fc9bf8be</t>
         </is>
       </c>
     </row>
@@ -1551,11 +1581,11 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>53698</v>
+        <v>84804</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>d2a60d2df159dd5773262648198d95fa05aa2dfc6b36ea5ca4208c6b7b421ed5</t>
+          <t>e76ef7bdd739d477778ddbb6fc7041afcc9fc3d9b292da5b92d1bd580c195934</t>
         </is>
       </c>
     </row>
@@ -1566,1389 +1596,1569 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1364872</v>
+        <v>1186676</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>deff101f038b17d4bd5a4545fd371aa0c588c56565c5238d555bfb4471899aa1</t>
+          <t>e5e1d869d315617342e7703e07263104717240eefe21046d9d6eaee2da0a0cac</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>outputs/figures/figure_bundle_audit.json</t>
+          <t>outputs/figures/FigD5_8_dimension_availability_sensitivity.pdf</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>2409</v>
+        <v>53301</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>da3ebd141c082e91a1745abc60394a9bc5c09de0cd31ad6297aa5cafc4d49756</t>
+          <t>49e7849bed2cbf5a3af29f9bfa72488baeb1f04a062c690e04d1a806be450f8c</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>outputs/local/D5_ablation_redundancy.xlsx</t>
+          <t>outputs/figures/FigD5_8_dimension_availability_sensitivity.png</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>9984</v>
+        <v>535313</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>f0feb1f3c9868bf39b167645436a3c13adea0cb6253ce840188905750b8c2157</t>
+          <t>25eed423cc1a6f55d00a2658d7ce4a3fd7a3e60bad1fdf6a6f6f4ff5cc3d51cb</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>outputs/local/D5_admission_decision.json</t>
+          <t>outputs/figures/FigD5_8_dimension_availability_sensitivity.svg</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>588</v>
+        <v>69730</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>a9c40d2d57897245afa23202d8e7ba49245ff63b19b9427ab86d12003a4c1583</t>
+          <t>9c9db61371e8dadf062ac4589057466d04d3164a6219d6ae0526685644ae2279</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>outputs/local/D5_admission_decision.xlsx</t>
+          <t>outputs/figures/FigD5_8_dimension_availability_sensitivity.tiff</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>6135</v>
+        <v>1406590</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>96cce073f38f1f8e9d436722f18513ea84f6acf4ba33920ca07d1185db5767dd</t>
+          <t>5e3895e9fe1ed2a5ad7e18aba0096ca11933e581e01f1cfc3cd65a08927cc045</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>outputs/local/D5_audit_log.xlsx</t>
+          <t>outputs/figures/FigD5_9_target_support_robustness.pdf</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>74702</v>
+        <v>48906</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>675cf312d5aa5e97cb8f722b22af3a9782c2b91a9dd3f12f708cfd6bb4955e3c</t>
+          <t>8967eaf6d8533c8a760b891ff04aa2f0a23251f9bbfb462bb6fddbf45c30a018</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>outputs/local/D5_case_study_exports.xlsx</t>
+          <t>outputs/figures/FigD5_9_target_support_robustness.png</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>44198</v>
+        <v>406917</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>060027cb3475620e45c16a5aed24ec4f94b00c01a7a3ba027a188963d7682dbc</t>
+          <t>fd0415d6e3ed87344cc5140186fd9b86626bfd1225dfd72662dae3042f1f5360</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>outputs/local/D5_edge_profile_summary.xlsx</t>
+          <t>outputs/figures/FigD5_9_target_support_robustness.svg</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>26857</v>
+        <v>35150</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>5b3bd2c7f60bb706732433cc146f79297976ea8f202150b40c281c932b3a6329</t>
+          <t>f8fdc6177a692a4ce6161c531314929cf6554203d8a30d815f015e6ec4eea8cd</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>outputs/local/D5_event_windows.parquet</t>
+          <t>outputs/figures/FigD5_9_target_support_robustness.tiff</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>80614</v>
+        <v>1040878</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2874ab1d42be1723d6baabd3bd81b768d9f4b3fcf5459712e226f029f25a24fd</t>
+          <t>88af281d37f8851618be048e49a8313a4a1a8a3a1e1d3f452a9b911daca6168d</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>outputs/local/D5_event_windows.xlsx</t>
+          <t>outputs/figures/figure_bundle_audit.json</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>140097</v>
+        <v>2409</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>97f101d88e4b67e9376735a772083ed8f1403eb700de6666b4a51314b7bc3dae</t>
+          <t>da3ebd141c082e91a1745abc60394a9bc5c09de0cd31ad6297aa5cafc4d49756</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>outputs/local/D5_gate_interface.parquet</t>
+          <t>outputs/local/D5_ablation_redundancy.xlsx</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>796803</v>
+        <v>9984</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>22b640fa64ff95f0677bdcafea1517c192dd506fc11559efc53db49916918e0e</t>
+          <t>f0feb1f3c9868bf39b167645436a3c13adea0cb6253ce840188905750b8c2157</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>outputs/local/D5_gate_interface.schema.json</t>
+          <t>outputs/local/D5_admission_decision.json</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>1128</v>
+        <v>588</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>619b0d9ef22475a5de39a752b479540987d05f9cb5d649e2f7bece38005622f3</t>
+          <t>a9c40d2d57897245afa23202d8e7ba49245ff63b19b9427ab86d12003a4c1583</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>outputs/local/D5_gate_interface.xlsx</t>
+          <t>outputs/local/D5_admission_decision.xlsx</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>5209423</v>
+        <v>6135</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>cc6458fcb96aa750a01b53bb7acfaceae4f832b53e68bd1840f57a8ee787b22c</t>
+          <t>96cce073f38f1f8e9d436722f18513ea84f6acf4ba33920ca07d1185db5767dd</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>outputs/local/D5_main_scores_hourly.parquet</t>
+          <t>outputs/local/D5_audit_log.xlsx</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>7340495</v>
+        <v>75667</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>64274562d7139d510dd3780dbd67bd2c2c5913908dbbec8ac7d4bcceb0418cd1</t>
+          <t>e6c5af19d0fc71dd80876b444f5272a8ca648d14ee9e8fbacfb99b71178a36a7</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>outputs/local/D5_main_scores_hourly.xlsx</t>
+          <t>outputs/local/D5_case_study_exports.xlsx</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>45272583</v>
+        <v>44198</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2ae0e3dcb195bddabcb98ac87479345348da28818c565a978c56f75ff0ee19c9</t>
+          <t>060027cb3475620e45c16a5aed24ec4f94b00c01a7a3ba027a188963d7682dbc</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>outputs/local/D5_mapping_params.xlsx</t>
+          <t>outputs/local/D5_edge_profile_summary.xlsx</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>20237</v>
+        <v>26857</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>30ffe256d465c57c614fcab9fa40d92fcd68a7c1f5fc78cbd8e0e0d00779b6a6</t>
+          <t>5b3bd2c7f60bb706732433cc146f79297976ea8f202150b40c281c932b3a6329</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>outputs/local/D5_multiscale_aggregates.xlsx</t>
+          <t>outputs/local/D5_event_windows.parquet</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>1060062</v>
+        <v>80614</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>96da07e011eecb169c1880e11e5c8656c9aa16a62434b3ad540a8b9a658a5da0</t>
+          <t>2874ab1d42be1723d6baabd3bd81b768d9f4b3fcf5459712e226f029f25a24fd</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>outputs/local/D5_reference_window_library.parquet</t>
+          <t>outputs/local/D5_event_windows.xlsx</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>62947</v>
+        <v>140097</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>b84bd8208e2e533e83c722868f022eaf87e07991f184e6d59e9411909e5360bc</t>
+          <t>97f101d88e4b67e9376735a772083ed8f1403eb700de6666b4a51314b7bc3dae</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>outputs/local/D5_reference_window_library.xlsx</t>
+          <t>outputs/local/D5_gate_interface.parquet</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>228952</v>
+        <v>796803</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>12bb084003accca5fd0e85f42191286a56a27c7016b617296cde45ff4004edf1</t>
+          <t>22b640fa64ff95f0677bdcafea1517c192dd506fc11559efc53db49916918e0e</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>outputs/local/D5_regime_state.parquet</t>
+          <t>outputs/local/D5_gate_interface.schema.json</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>3658910</v>
+        <v>1128</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>622dd0f5ed1473ae5de464e4207e51ff9470de209cadcee9b30cbac92f9392e8</t>
+          <t>619b0d9ef22475a5de39a752b479540987d05f9cb5d649e2f7bece38005622f3</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>outputs/local/D5_regime_state.xlsx</t>
+          <t>outputs/local/D5_gate_interface.xlsx</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>45834835</v>
+        <v>5209423</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>427fe81df8b7861210e267f694058376a754fa724e0bbafe1b07208e32787485</t>
+          <t>cc6458fcb96aa750a01b53bb7acfaceae4f832b53e68bd1840f57a8ee787b22c</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>outputs/local/D5_report_interface.parquet</t>
+          <t>outputs/local/D5_main_scores_hourly.parquet</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>1171194</v>
+        <v>7340495</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>f057e0a8037282fb43a71a94d7043c7bd3de2b4c8fa9865365bcf0427195dbda</t>
+          <t>64274562d7139d510dd3780dbd67bd2c2c5913908dbbec8ac7d4bcceb0418cd1</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>outputs/local/D5_report_interface.schema.json</t>
+          <t>outputs/local/D5_main_scores_hourly.xlsx</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>853</v>
+        <v>45272583</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>c740ff5a12c99a1a761c5f2ab45d12f5174aaac3b2201e58e6d67a1a8c87c06e</t>
+          <t>2ae0e3dcb195bddabcb98ac87479345348da28818c565a978c56f75ff0ee19c9</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>outputs/local/D5_report_interface.xlsx</t>
+          <t>outputs/local/D5_mapping_params.xlsx</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>11410677</v>
+        <v>20237</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>f9040450b3fb8204f2fea44f92c003d1cdc2acf900a29715ee732a8b9b450aae</t>
+          <t>30ffe256d465c57c614fcab9fa40d92fcd68a7c1f5fc78cbd8e0e0d00779b6a6</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>outputs/local/D5_sensor_influence.parquet</t>
+          <t>outputs/local/D5_multiscale_aggregates.xlsx</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>6011187</v>
+        <v>1060062</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>a9270494760fcb4ae501abcf54c50e813ca74d6306d7fbca94d7ef1a1d1730a2</t>
+          <t>96da07e011eecb169c1880e11e5c8656c9aa16a62434b3ad540a8b9a658a5da0</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>outputs/local/D5_sensor_influence.xlsx</t>
+          <t>outputs/local/D5_reference_window_library.parquet</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>16403976</v>
+        <v>62947</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>338920c1db9c7b1bc500fa43d92f02f6165187545a79f696771287bfd877a9a0</t>
+          <t>b84bd8208e2e533e83c722868f022eaf87e07991f184e6d59e9411909e5360bc</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>outputs/local/D5_sensor_profile_summary.xlsx</t>
+          <t>outputs/local/D5_reference_window_library.xlsx</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>7442</v>
+        <v>228952</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>aef38bd66378a9ae3b2c76a848f1ef4d51d504616c435440e45f99eadf9fb5a9</t>
+          <t>12bb084003accca5fd0e85f42191286a56a27c7016b617296cde45ff4004edf1</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>outputs/local/D5_spatial_evidence.parquet</t>
+          <t>outputs/local/D5_regime_state.parquet</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>6146048</v>
+        <v>3658910</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>4edb2bd1af0cbdac8fc61382508099137349f67f6ce70da4ee1831848bfe3733</t>
+          <t>622dd0f5ed1473ae5de464e4207e51ff9470de209cadcee9b30cbac92f9392e8</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>outputs/local/D5_spatial_evidence.xlsx</t>
+          <t>outputs/local/D5_regime_state.xlsx</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>15958642</v>
+        <v>45834835</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>6e2a433bcdb115b841f269c5eb5184623502c7221234da51b8ade0377c120327</t>
+          <t>427fe81df8b7861210e267f694058376a754fa724e0bbafe1b07208e32787485</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>outputs/local/D5_spatial_templates.template_bundle.json</t>
+          <t>outputs/local/D5_report_interface.parquet</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>542571</v>
+        <v>1171194</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>704238fcb5551593e569bdb3e015f04cb710815fdeccbb8aa28ba9a0c7e59ace</t>
+          <t>f057e0a8037282fb43a71a94d7043c7bd3de2b4c8fa9865365bcf0427195dbda</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>outputs/local/D5_spatial_templates.xlsx</t>
+          <t>outputs/local/D5_report_interface.schema.json</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>190694</v>
+        <v>853</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>6fc3291e19dd0663ccd33db897edbf39e67f54e7db7b1fa8de0648d06d82c6bc</t>
+          <t>c740ff5a12c99a1a761c5f2ab45d12f5174aaac3b2201e58e6d67a1a8c87c06e</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>outputs/local/D5_support_assessment.parquet</t>
+          <t>outputs/local/D5_report_interface.xlsx</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>52815</v>
+        <v>11410677</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>00d3ed69dc3899db48c841bb56c6664bc1832e365fd5fa5c13130b6d231e5750</t>
+          <t>f9040450b3fb8204f2fea44f92c003d1cdc2acf900a29715ee732a8b9b450aae</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>outputs/local/D5_support_assessment.xlsx</t>
+          <t>outputs/local/D5_sensor_influence.parquet</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>28036</v>
+        <v>6011187</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>34df65d8e4329d166c69a9bc505bb97a8397e537f323c5be392fba093827dd98</t>
+          <t>a9270494760fcb4ae501abcf54c50e813ca74d6306d7fbca94d7ef1a1d1730a2</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>outputs/local/D5_topology_drift_alerts.parquet</t>
+          <t>outputs/local/D5_sensor_influence.xlsx</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>10824</v>
+        <v>16403976</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>59d05a6c138fc18e295611bb0e39f469c07f6a25522ed809ea4f76ca018a908a</t>
+          <t>338920c1db9c7b1bc500fa43d92f02f6165187545a79f696771287bfd877a9a0</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>outputs/local/D5_topology_drift_alerts.xlsx</t>
+          <t>outputs/local/D5_sensor_profile_summary.xlsx</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>9965</v>
+        <v>7442</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>7262caaddcf1713a512e6dd52157f3f0e4bee9ae2642dcaf63eed60ff9ce9a87</t>
+          <t>aef38bd66378a9ae3b2c76a848f1ef4d51d504616c435440e45f99eadf9fb5a9</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>outputs/local/D5_topology_evidence.yaml</t>
+          <t>outputs/local/D5_spatial_evidence.parquet</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>2342</v>
+        <v>6146048</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>50abd276a9e6bbf26acb9a22d3a796ca63423d363a036422dc57c6bdfeb71920</t>
+          <t>4edb2bd1af0cbdac8fc61382508099137349f67f6ce70da4ee1831848bfe3733</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>outputs/local/D5_topology_registry.json</t>
+          <t>outputs/local/D5_spatial_evidence.xlsx</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>14821</v>
+        <v>15958642</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>6efbf6722e2caecabf2d9999637d48bbb7c4d630dc3e9354982ed89d750965bc</t>
+          <t>6e2a433bcdb115b841f269c5eb5184623502c7221234da51b8ade0377c120327</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>outputs/local/D5_topology_registry.schema.json</t>
+          <t>outputs/local/D5_spatial_templates.template_bundle.json</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>1301</v>
+        <v>542571</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>0f4c6e9e6d510996d1435efd1810b4a1eaca35a989b7f3d78187e29f8ce9584e</t>
+          <t>704238fcb5551593e569bdb3e015f04cb710815fdeccbb8aa28ba9a0c7e59ace</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>outputs/local/D5_topology_registry.xlsx</t>
+          <t>outputs/local/D5_spatial_templates.xlsx</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>11679</v>
+        <v>190694</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>7aa5db4087c2346acc99d827f7c3a0bd49ce90540fb2ec8f56664c82b14e36ff</t>
+          <t>6fc3291e19dd0663ccd33db897edbf39e67f54e7db7b1fa8de0648d06d82c6bc</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>outputs/local/D5_topology_registry.yaml</t>
+          <t>outputs/local/D5_support_assessment.parquet</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>2838</v>
+        <v>52815</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>46e191549a0c768ee947bff4d98f26f38a93ecbce380ab4ff8114d2885dd29f9</t>
+          <t>00d3ed69dc3899db48c841bb56c6664bc1832e365fd5fa5c13130b6d231e5750</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>outputs/local/D5_validation_results.xlsx</t>
+          <t>outputs/local/D5_support_assessment.xlsx</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>64326</v>
+        <v>28036</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>b4a0f5586b1108b945dba84b87a47a7f387c11fa182de0c506977f3c9870efff</t>
+          <t>34df65d8e4329d166c69a9bc505bb97a8397e537f323c5be392fba093827dd98</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>outputs/local/D5_zone_consensus.parquet</t>
+          <t>outputs/local/D5_topology_drift_alerts.parquet</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>1618880</v>
+        <v>10824</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>0cb43651f4dc8c4a7f378cfe3be964a688e7df7a2ff45052f649259b415cdb8c</t>
+          <t>59d05a6c138fc18e295611bb0e39f469c07f6a25522ed809ea4f76ca018a908a</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>outputs/local/D5_zone_consensus.xlsx</t>
+          <t>outputs/local/D5_topology_drift_alerts.xlsx</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>7277838</v>
+        <v>9965</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>f43c5554c5a0c9f3e50e38f51bc0db270a9c819c3a00a9f3dc23ae658b7e7149</t>
+          <t>7262caaddcf1713a512e6dd52157f3f0e4bee9ae2642dcaf63eed60ff9ce9a87</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>outputs/plot_data/D5_plot_data.csv</t>
+          <t>outputs/local/D5_topology_evidence.yaml</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>18506701</v>
+        <v>2342</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>f074d7394f60df5f9b874734fe644757863bf44e876dd97303344227afe065c3</t>
+          <t>50abd276a9e6bbf26acb9a22d3a796ca63423d363a036422dc57c6bdfeb71920</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>outputs/plot_data/D5_plot_data.parquet</t>
+          <t>outputs/local/D5_topology_registry.json</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>744459</v>
+        <v>14821</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>3236229f520cfa38329877aa013a7233229a77567e32c95b37a87d5fe94a5dd8</t>
+          <t>6efbf6722e2caecabf2d9999637d48bbb7c4d630dc3e9354982ed89d750965bc</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>outputs/plot_data/D5_plot_data_manifest.json</t>
+          <t>outputs/local/D5_topology_registry.schema.json</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>519</v>
+        <v>1301</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>27ae5a05d462aab27e6a6359daaf99d931840e8b58d462da108ff3ca12dfc1ae</t>
+          <t>0f4c6e9e6d510996d1435efd1810b4a1eaca35a989b7f3d78187e29f8ce9584e</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>outputs/publication/D5_coverage_strata.parquet</t>
+          <t>outputs/local/D5_topology_registry.xlsx</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>5837</v>
+        <v>11679</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>f4da589996c29b4e710131be262c3efdaa0fb822e051293f1310365aaf0e7b75</t>
+          <t>7aa5db4087c2346acc99d827f7c3a0bd49ce90540fb2ec8f56664c82b14e36ff</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>outputs/publication/D5_coverage_summary.parquet</t>
+          <t>outputs/local/D5_topology_registry.yaml</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>2879</v>
+        <v>2838</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>54201e6be7009f8ed97eb53e8abd9d8d33766757486839e1d1650d09bf1718c6</t>
+          <t>46e191549a0c768ee947bff4d98f26f38a93ecbce380ab4ff8114d2885dd29f9</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>outputs/publication/D5_d4_d5_composite.parquet</t>
+          <t>outputs/local/D5_validation_results.xlsx</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>4352</v>
+        <v>64326</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>54eed66c77212702829f3d4bc85907babd66e415997082a0a86a8b49ea1b4556</t>
+          <t>b4a0f5586b1108b945dba84b87a47a7f387c11fa182de0c506977f3c9870efff</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>outputs/publication/D5_d4_d5_dependence.parquet</t>
+          <t>outputs/local/D5_zone_consensus.parquet</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>4364</v>
+        <v>1618880</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>a18b2d57e0affd0fdf036d32f43b988f92c6866b4300aa8cfa798991759f1268</t>
+          <t>0cb43651f4dc8c4a7f378cfe3be964a688e7df7a2ff45052f649259b415cdb8c</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>outputs/publication/D5_decision_register.parquet</t>
+          <t>outputs/local/D5_zone_consensus.xlsx</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>4691</v>
+        <v>7277838</v>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>8c888a1b2a0a3790d1333395853deb23b7c145c3a9489c8464c595fef28427f9</t>
+          <t>f43c5554c5a0c9f3e50e38f51bc0db270a9c819c3a00a9f3dc23ae658b7e7149</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>outputs/publication/D5_localization.parquet</t>
+          <t>outputs/plot_data/D5_plot_data.csv</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>6980</v>
+        <v>18506701</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>e63682e2c8a0ebeb772d9d0eae21b4be654b370f853eb939376249c595ddfcff</t>
+          <t>f074d7394f60df5f9b874734fe644757863bf44e876dd97303344227afe065c3</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>outputs/publication/D5_monthly_coverage.parquet</t>
+          <t>outputs/plot_data/D5_plot_data.parquet</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>6919</v>
+        <v>744459</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>51e4fd571650b85d5e4d8c2aab7c0ca543cb81aff01517a7efacc70c08bea506</t>
+          <t>3236229f520cfa38329877aa013a7233229a77567e32c95b37a87d5fe94a5dd8</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>outputs/publication/D5_outer_refit_deltas.parquet</t>
+          <t>outputs/plot_data/D5_plot_data_manifest.json</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>7921</v>
+        <v>519</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>1601955bc59dfd0da87cd33e695f16ac974ad0be8ecacbdb23dfe465599ce7bf</t>
+          <t>27ae5a05d462aab27e6a6359daaf99d931840e8b58d462da108ff3ca12dfc1ae</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>outputs/publication/D5_outer_refit_summary.parquet</t>
+          <t>outputs/publication/D5_coverage_strata.parquet</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>6681</v>
+        <v>5837</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>9ea7de7e9e34e2bc3b5c657dd72bded594918e0310ad7e231a2610ef45253f30</t>
+          <t>f4da589996c29b4e710131be262c3efdaa0fb822e051293f1310365aaf0e7b75</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>outputs/publication/D5_publication_audit_manifest.json</t>
+          <t>outputs/publication/D5_coverage_summary.parquet</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>4364</v>
+        <v>2879</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>e3fb4bafbf07c9310f2c5afae1737d00b609f7d8c0f563b1d51366aab2cd3df3</t>
+          <t>54201e6be7009f8ed97eb53e8abd9d8d33766757486839e1d1650d09bf1718c6</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>outputs/publication/D5_publication_audit_tables.xlsx</t>
+          <t>outputs/publication/D5_d4_d5_composite.parquet</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>23665</v>
+        <v>4352</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>f804b0704ef36c432f26f3faf80d6ad7cbf93f014ec02a34916644a509ae3dae</t>
+          <t>54eed66c77212702829f3d4bc85907babd66e415997082a0a86a8b49ea1b4556</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>outputs/publication/D5_PUBLICATION_READINESS_AUDIT_v1.0.md</t>
+          <t>outputs/publication/D5_d4_d5_dependence.parquet</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>5709</v>
+        <v>5734</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>951b14afceb659a941306c90c0763fec61bf79de8cd0d5316024059cfbdf7bdf</t>
+          <t>5a460deb7c3336af77955fa2de04d3386bb208a978ec8998174b14ce2f505fa3</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>outputs/publication/D5_risk_coverage.parquet</t>
+          <t>outputs/publication/D5_d4_d5_stratified_rho.parquet</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>5064</v>
+        <v>8751</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>eb0caf68ddfdc8203a64254c3aa277304432bb3fa762cb19e0b9123740a49508</t>
+          <t>4e274bbb6e5a161f0079a012dd37cdd2d20d7558f1b2e2ac004d56269c814ddd</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>outputs/publication/D5_support_sensitivity.parquet</t>
+          <t>outputs/publication/D5_decision_register.parquet</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>5871</v>
+        <v>4974</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>f6ee73f3893ed53682e63122e9220948cc97ffa0c9ead47b20b6b2c739de9fda</t>
+          <t>710460457bcba4163b5d64d66b94ca476495f41a95378efddd2581ffa32a0196</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>outputs/publication/D5_target_influence.parquet</t>
+          <t>outputs/publication/D5_dimension_availability.parquet</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>8536</v>
+        <v>12550</v>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>77b6a0a69423e32f3f664790ccd0b4e841d967fce6370559b159ea50c758bdad</t>
+          <t>f34750499b681fb5eefe3f811fbbec3a4d0570f45ca71a850a191b4a67c93680</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>outputs/publication/FigD5_6_validation_coverage_source_data.xlsx</t>
+          <t>outputs/publication/D5_localization.parquet</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>10606</v>
+        <v>6980</v>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>12a62815cd1300db24c3c293d091547a95a521a3b965009db4e36ff41493ada4</t>
+          <t>e63682e2c8a0ebeb772d9d0eae21b4be654b370f853eb939376249c595ddfcff</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>outputs/publication/FigD5_7_D4_D5_complementarity_source_data.xlsx</t>
+          <t>outputs/publication/D5_monthly_coverage.parquet</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>9134</v>
+        <v>6919</v>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>325b0094eb3ea93567482e7648b5740f141441b830fd2e540c5805c3120d5d52</t>
+          <t>51e4fd571650b85d5e4d8c2aab7c0ca543cb81aff01517a7efacc70c08bea506</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_CURRENT_RELEASE.md</t>
+          <t>outputs/publication/D5_outer_refit_deltas.parquet</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>916</v>
+        <v>7921</v>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>de2a0d79f1cc37684c35cae1e61858482c4476d9951c724a1c28dd40af6c44d1</t>
+          <t>1601955bc59dfd0da87cd33e695f16ac974ad0be8ecacbdb23dfe465599ce7bf</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_EXPERT_REPORT_v2.1.docx</t>
+          <t>outputs/publication/D5_outer_refit_summary.parquet</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>2047657</v>
+        <v>6681</v>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>8e5db363b70bd05b8584eb191b764d1d2beee31c2be738b56f44c9902c67fb04</t>
+          <t>9ea7de7e9e34e2bc3b5c657dd72bded594918e0310ad7e231a2610ef45253f30</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_EXPERT_REPORT_v2.1.md</t>
+          <t>outputs/publication/D5_publication_audit_manifest.json</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>7814</v>
+        <v>10292</v>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>6de0e55c9c7f57f2c030d48076b3da316a94d53167e1c1e9d164031972691657</t>
+          <t>5e18a160b4c90f186cc654abc505b2ee64abf30c70e3b7d4f659340665bb8336</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_EXPERT_REPORT_v2.2.docx</t>
+          <t>outputs/publication/D5_publication_audit_tables.xlsx</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>2107226</v>
+        <v>30537</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>9dfbe96a145765a0e22e8452ec1a76f759ae52cd201b71694aa7c7e815fd8d8b</t>
+          <t>600e9aefde2898da31fc87ba4ca5d2878324ba73ec76f2b6b0d4704887c36794</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_EXPERT_REPORT_v2.2.md</t>
+          <t>outputs/publication/D5_PUBLICATION_READINESS_AUDIT_v1.1.md</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>8480</v>
+        <v>7400</v>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>5f9333b22a9d8dc1b40d9ac2f1f684ee851785bf1f742be406e6433cfc841cfd</t>
+          <t>3000fd27bd303e5413d1d7eb5b5d7a464ac2e416930890be51a8a1928182ab5f</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_EXPERT_REPORT_v2.3.docx</t>
+          <t>outputs/publication/D5_risk_coverage.parquet</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>2056532</v>
+        <v>5064</v>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>19b15492f9b09b02820cf4ff0effd41c672a7dd0a99a42eef3886c732b622fe5</t>
+          <t>eb0caf68ddfdc8203a64254c3aa277304432bb3fa762cb19e0b9123740a49508</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_EXPERT_REPORT_v2.3.md</t>
+          <t>outputs/publication/D5_support_sensitivity.parquet</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>9043</v>
+        <v>5871</v>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>93baa7ffe8d1d92abac60ce6896dd742d71410bb89c771ab5d8e73c9bc3d6b57</t>
+          <t>f6ee73f3893ed53682e63122e9220948cc97ffa0c9ead47b20b6b2c739de9fda</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_EXPERT_REPORT_v2.4.docx</t>
+          <t>outputs/publication/D5_target_influence.parquet</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>3111730</v>
+        <v>8537</v>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>cc1e9c76ec52cffba4e49f71fddbcc746efd6c195e41cfda57373264bd57078b</t>
+          <t>13af4a843ab3f1942fe634e88b6bb8badd884917e8a2533d602bff89b59f54ff</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_EXPERT_REPORT_v2.4.md</t>
+          <t>outputs/publication/FigD5_6_validation_coverage_source_data.xlsx</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>9532</v>
+        <v>10606</v>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>fc5b363eb632924c649f82b46c9848f77eff3e0f4a430ceedd119e5b7542426c</t>
+          <t>c3a6003ecea1362dab936bfbad45fc6ef37294636555b31a7aa505186cff8080</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_FIGURE_CAPTIONS_v2.1.md</t>
+          <t>outputs/publication/FigD5_7_D4_D5_complementarity_source_data.xlsx</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>2282</v>
+        <v>10601</v>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>dd5ca9eea1365f682a5166e6f8e11da3da1b6ce06652795ba6bd0112a5711bc0</t>
+          <t>8c27e8a3c215ea325839dc203b968a69582e270588e1d5bb0fca1759624c4210</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_FIGURE_CAPTIONS_v2.2.md</t>
+          <t>outputs/publication/FigD5_8_dimension_availability_sensitivity_source_data.xlsx</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>2185</v>
+        <v>6490</v>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>4e3e50df15c243b7c789337fb51e9fe8f350c3815f05b408b6dd2f8aad9c4067</t>
+          <t>7619005d9470f6485750c452ea79fcfbff717ebab60ac2fb072170b5be2dd583</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_FIGURE_CAPTIONS_v2.3.md</t>
+          <t>outputs/publication/FigD5_9_target_support_robustness_source_data.xlsx</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>2471</v>
+        <v>7501</v>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>5aace3b407bf260ee6a54a95a25736b01d1ec2831a95823a45288d40270b532c</t>
+          <t>300a6cb9e7b6f8c6c8ef1f043ddea916673046772105d1209cb6d9b1dbcabf3c</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_FIGURE_CAPTIONS_v2.4.md</t>
+          <t>outputs/reports/D5_CURRENT_RELEASE.md</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>3600</v>
+        <v>1075</v>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>555abddc4fd206f1d6afe947be1fad9f7557a5162e37116fa4537fd8fcc087bb</t>
+          <t>51b1250c4db8d4e2fc5fa97b2ebe2da15e4e47b37d9de1f8097b4e24b148ad20</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_PROJECT_DIRECTORY_GUIDE_v2.1.docx</t>
+          <t>outputs/reports/D5_EXPERT_REPORT_v2.1.docx</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>40336</v>
+        <v>2047657</v>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>c2da3e9cca5ef0a5e83b63089e8deeb7299a7e0e7735c0b4751cd47f2fc47844</t>
+          <t>8e5db363b70bd05b8584eb191b764d1d2beee31c2be738b56f44c9902c67fb04</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_PROJECT_DIRECTORY_GUIDE_v2.1.md</t>
+          <t>outputs/reports/D5_EXPERT_REPORT_v2.1.md</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>5333</v>
+        <v>7814</v>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>0303a5bbdc16689493eb5b3826d95bf7c23fc4405284ef7db01d13b5a1d1b045</t>
+          <t>6de0e55c9c7f57f2c030d48076b3da316a94d53167e1c1e9d164031972691657</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_PROJECT_DIRECTORY_GUIDE_v2.2.docx</t>
+          <t>outputs/reports/D5_EXPERT_REPORT_v2.2.docx</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>40363</v>
+        <v>2107226</v>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>eada32c51f435a6355dc873b748b4f894cbbc17bedfc4be6090371aa323aea5e</t>
+          <t>9dfbe96a145765a0e22e8452ec1a76f759ae52cd201b71694aa7c7e815fd8d8b</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_PROJECT_DIRECTORY_GUIDE_v2.2.md</t>
+          <t>outputs/reports/D5_EXPERT_REPORT_v2.2.md</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>5307</v>
+        <v>8480</v>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>b63d3b48b8902ad31fcbeac70f218c2c3abd2b1ee4293aff45cbc89fe16b950b</t>
+          <t>5f9333b22a9d8dc1b40d9ac2f1f684ee851785bf1f742be406e6433cfc841cfd</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_PROJECT_DIRECTORY_GUIDE_v2.3.docx</t>
+          <t>outputs/reports/D5_EXPERT_REPORT_v2.3.docx</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>40364</v>
+        <v>2056532</v>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>788d71134331e7d994e157cbfb511ef1f5966eb546d05ea3a77a8b2dd90c2fce</t>
+          <t>19b15492f9b09b02820cf4ff0effd41c672a7dd0a99a42eef3886c732b622fe5</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_PROJECT_DIRECTORY_GUIDE_v2.3.md</t>
+          <t>outputs/reports/D5_EXPERT_REPORT_v2.3.md</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>5459</v>
+        <v>9043</v>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>0308ed8c677cbbb3581e4022bbc99623af3de79cf83fc9283b160fd54cb8d503</t>
+          <t>93baa7ffe8d1d92abac60ce6896dd742d71410bb89c771ab5d8e73c9bc3d6b57</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_PROJECT_DIRECTORY_GUIDE_v2.4.docx</t>
+          <t>outputs/reports/D5_EXPERT_REPORT_v2.4.docx</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>40366</v>
+        <v>3904525</v>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>3306d9a6afcb510e296a5c9031cbe916a059fb0c52e6431ad4ac8d67bf146f58</t>
+          <t>555acc56c3cbff9e389ab77b43e570a75b916697e57efb691387db00be069c2e</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_PROJECT_DIRECTORY_GUIDE_v2.4.md</t>
+          <t>outputs/reports/D5_EXPERT_REPORT_v2.4.md</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>5670</v>
+        <v>10252</v>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>f68468aa772b22e9fd44f55c62997fa53699339f963e6de09346c7a502fec34e</t>
+          <t>1bc7c85d339d3df9deb1c08eafe0aa8b0b9c7d5e81a30b9e41ef39cfa4dbbd45</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>outputs/reports/nature_figure_bundle_audit.json</t>
+          <t>outputs/reports/D5_FIGURE_CAPTIONS_v2.1.md</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>2409</v>
+        <v>2282</v>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>da3ebd141c082e91a1745abc60394a9bc5c09de0cd31ad6297aa5cafc4d49756</t>
+          <t>dd5ca9eea1365f682a5166e6f8e11da3da1b6ce06652795ba6bd0112a5711bc0</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>outputs/sensitivity/D5_sensitivity_manifest.json</t>
+          <t>outputs/reports/D5_FIGURE_CAPTIONS_v2.2.md</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>2345</v>
+        <v>2185</v>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>71ddb925f1c43c2bb363be78cb221f6a90ed9d1bce2beb713989957efcb0b8d8</t>
+          <t>4e3e50df15c243b7c789337fb51e9fe8f350c3815f05b408b6dd2f8aad9c4067</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>outputs/sensitivity/D5_shadow_scores.parquet</t>
+          <t>outputs/reports/D5_FIGURE_CAPTIONS_v2.3.md</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>2987712</v>
+        <v>2471</v>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>a54b95d4cada7ab1f9a1e4bd7723d29f46c9e3c19de2bcab6f52a9da161ba5fc</t>
+          <t>5aace3b407bf260ee6a54a95a25736b01d1ec2831a95823a45288d40270b532c</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>outputs/sensitivity/D5_shadow_scores.xlsx</t>
+          <t>outputs/reports/D5_FIGURE_CAPTIONS_v2.4.md</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>10004039</v>
+        <v>4620</v>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>1229f93be5258226bfbdc36daab2ceb3aa2b475485c1fa0392cc15ec148a97f9</t>
+          <t>8eebf74993e5b086730cf83b7953f1ae363c9e94dc2eb38ec7d3475a28496094</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>outputs/sensitivity/D5_shadow_template_shift.xlsx</t>
+          <t>outputs/reports/D5_PROJECT_DIRECTORY_GUIDE_v2.1.docx</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>41680</v>
+        <v>40336</v>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>3f68e2e6f4d6bc46aa021613f6b8ee25bb562d0798f1896ef47555b36c89fe35</t>
+          <t>c2da3e9cca5ef0a5e83b63089e8deeb7299a7e0e7735c0b4751cd47f2fc47844</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>outputs/sensitivity/D5_track_invariance.xlsx</t>
+          <t>outputs/reports/D5_PROJECT_DIRECTORY_GUIDE_v2.1.md</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>14538</v>
+        <v>5333</v>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>c9ed72b9a91d1fa854692c1cabf77687a652bf9723a7d405b4fbc08cf5b6c1c0</t>
+          <t>0303a5bbdc16689493eb5b3826d95bf7c23fc4405284ef7db01d13b5a1d1b045</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>outputs/shadow_v2/D5_graph_structure_learning_shadow.parquet</t>
+          <t>outputs/reports/D5_PROJECT_DIRECTORY_GUIDE_v2.2.docx</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>9388</v>
+        <v>40363</v>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>f65546587bfb8c5a13efa5af7a38f57820bb3467cbd974c3bfad3c369a88f2c7</t>
+          <t>eada32c51f435a6355dc873b748b4f894cbbc17bedfc4be6090371aa323aea5e</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>outputs/shadow_v2/D5_graph_structure_learning_shadow.xlsx</t>
+          <t>outputs/reports/D5_PROJECT_DIRECTORY_GUIDE_v2.2.md</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>8325</v>
+        <v>5307</v>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>b5a4109a1f1e707a2bc54497df9a808bd01cf23a9094aed4a77ff885fef49653</t>
+          <t>b63d3b48b8902ad31fcbeac70f218c2c3abd2b1ee4293aff45cbc89fe16b950b</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
+          <t>outputs/reports/D5_PROJECT_DIRECTORY_GUIDE_v2.3.docx</t>
+        </is>
+      </c>
+      <c r="B123" t="n">
+        <v>40364</v>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>788d71134331e7d994e157cbfb511ef1f5966eb546d05ea3a77a8b2dd90c2fce</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>outputs/reports/D5_PROJECT_DIRECTORY_GUIDE_v2.3.md</t>
+        </is>
+      </c>
+      <c r="B124" t="n">
+        <v>5459</v>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>0308ed8c677cbbb3581e4022bbc99623af3de79cf83fc9283b160fd54cb8d503</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>outputs/reports/D5_PROJECT_DIRECTORY_GUIDE_v2.4.docx</t>
+        </is>
+      </c>
+      <c r="B125" t="n">
+        <v>40394</v>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>87c9c02f45ee2222bed152e5932338f8c4970970af051579544d809c7118d5c8</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>outputs/reports/D5_PROJECT_DIRECTORY_GUIDE_v2.4.md</t>
+        </is>
+      </c>
+      <c r="B126" t="n">
+        <v>5732</v>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>b7d9a57e289f30d49b4a1d54acb47d2d49b883b3d55ea7113af8ec21f836baf1</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>outputs/reports/nature_figure_bundle_audit.json</t>
+        </is>
+      </c>
+      <c r="B127" t="n">
+        <v>2409</v>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>da3ebd141c082e91a1745abc60394a9bc5c09de0cd31ad6297aa5cafc4d49756</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>outputs/sensitivity/D5_sensitivity_manifest.json</t>
+        </is>
+      </c>
+      <c r="B128" t="n">
+        <v>2345</v>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>71ddb925f1c43c2bb363be78cb221f6a90ed9d1bce2beb713989957efcb0b8d8</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>outputs/sensitivity/D5_shadow_scores.parquet</t>
+        </is>
+      </c>
+      <c r="B129" t="n">
+        <v>2987712</v>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>a54b95d4cada7ab1f9a1e4bd7723d29f46c9e3c19de2bcab6f52a9da161ba5fc</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>outputs/sensitivity/D5_shadow_scores.xlsx</t>
+        </is>
+      </c>
+      <c r="B130" t="n">
+        <v>10004039</v>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>1229f93be5258226bfbdc36daab2ceb3aa2b475485c1fa0392cc15ec148a97f9</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>outputs/sensitivity/D5_shadow_template_shift.xlsx</t>
+        </is>
+      </c>
+      <c r="B131" t="n">
+        <v>41680</v>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>3f68e2e6f4d6bc46aa021613f6b8ee25bb562d0798f1896ef47555b36c89fe35</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>outputs/sensitivity/D5_track_invariance.xlsx</t>
+        </is>
+      </c>
+      <c r="B132" t="n">
+        <v>14538</v>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>c9ed72b9a91d1fa854692c1cabf77687a652bf9723a7d405b4fbc08cf5b6c1c0</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>outputs/shadow_v2/D5_graph_structure_learning_shadow.parquet</t>
+        </is>
+      </c>
+      <c r="B133" t="n">
+        <v>9388</v>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>f65546587bfb8c5a13efa5af7a38f57820bb3467cbd974c3bfad3c369a88f2c7</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>outputs/shadow_v2/D5_graph_structure_learning_shadow.xlsx</t>
+        </is>
+      </c>
+      <c r="B134" t="n">
+        <v>8325</v>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>b5a4109a1f1e707a2bc54497df9a808bd01cf23a9094aed4a77ff885fef49653</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
           <t>outputs/shadow_v2/D5_shadow_v2_manifest.json</t>
         </is>
       </c>
-      <c r="B123" t="n">
+      <c r="B135" t="n">
         <v>263</v>
       </c>
-      <c r="C123" t="inlineStr">
+      <c r="C135" t="inlineStr">
         <is>
           <t>b031365e134ba1bfee32dd92c04e35cdff1e904f78937c214e008540551a11f3</t>
         </is>

</xml_diff>

<commit_message>
Refresh D5 release audit metadata
</commit_message>
<xml_diff>
--- a/Project 1 Data Quality Assessment/D5 Topological Role Consistency and Structural Representativeness/outputs/local/D5_audit_log.xlsx
+++ b/Project 1 Data Quality Assessment/D5 Topological Role Consistency and Structural Representativeness/outputs/local/D5_audit_log.xlsx
@@ -1165,7 +1165,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2996a12d5c57570b074196dd8036c29032857b9fde93df7aea352aa371992c38</t>
+          <t>817b400fa63e6fab3ed0b096e5dd1c4d3e5b181c912be27e6dec22582da6ad1c</t>
         </is>
       </c>
     </row>
@@ -1791,11 +1791,11 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>75667</v>
+        <v>75669</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>e6c5af19d0fc71dd80876b444f5272a8ca648d14ee9e8fbacfb99b71178a36a7</t>
+          <t>bf0f605340ce0ce33a4bc9a3dd952bf55372ffa03a501a471da7472f9fe74554</t>
         </is>
       </c>
     </row>
@@ -2571,11 +2571,11 @@
         </is>
       </c>
       <c r="B96" t="n">
-        <v>10292</v>
+        <v>10358</v>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>5e18a160b4c90f186cc654abc505b2ee64abf30c70e3b7d4f659340665bb8336</t>
+          <t>a6ea3da8d8d0928abbf9557443849e45ce01a97f2d7df368fc8c8c5c3a548501</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bind D5 publication artifacts to frozen D4
</commit_message>
<xml_diff>
--- a/Project 1 Data Quality Assessment/D5 Topological Role Consistency and Structural Representativeness/outputs/local/D5_audit_log.xlsx
+++ b/Project 1 Data Quality Assessment/D5 Topological Role Consistency and Structural Representativeness/outputs/local/D5_audit_log.xlsx
@@ -775,11 +775,11 @@
         </is>
       </c>
       <c r="B16" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>exact single D4 run/calibration and main-score SHA-256; status=stale_dependency_blocked</t>
+          <t>exact single D4 run/calibration and main-score SHA-256; status=current</t>
         </is>
       </c>
     </row>
@@ -1161,11 +1161,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>28805</v>
+        <v>28550</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>817b400fa63e6fab3ed0b096e5dd1c4d3e5b181c912be27e6dec22582da6ad1c</t>
+          <t>83aa7ba54fb6d2e9499c22134ddc210a67a151f8526abb6304ba2c0c8f992802</t>
         </is>
       </c>
     </row>
@@ -1180,7 +1180,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>cfc1b4c9f71d05af39a974ef9463f90f52066b9e042c8f67b0930bec652f478f</t>
+          <t>6197278780f24a12047422d29727861d98c8487defc691e4a60bb3bb50cf9b5a</t>
         </is>
       </c>
     </row>
@@ -1495,7 +1495,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ff8beec018d4d331224ef2236e7fbe172b41f929f356e23c19359572ec4fb2e3</t>
+          <t>bd8b424c251d78568c23fd1dee1f0804d3cd0966daca1fbd5fdbf540df016cbb</t>
         </is>
       </c>
     </row>
@@ -1525,7 +1525,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>60ed8eabe554b2a7c014a37929d2a8c0a6cf9253c107e31f49657ac47e37352b</t>
+          <t>5b19aa268856963bd00229b76088adc9675c3a3436dcb4085c05db3c61cb0953</t>
         </is>
       </c>
     </row>
@@ -1551,11 +1551,11 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>58126</v>
+        <v>58200</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>1fc0731d8363ad2cc56a344a8b3410c920a9f51d34c938199548bfd4ef4d10a3</t>
+          <t>8a1bd5a137ec759b81994ef7e9551cf10bd2c81477915a64adc2ca1831f50ff3</t>
         </is>
       </c>
     </row>
@@ -1566,11 +1566,11 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>556320</v>
+        <v>590625</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>f4ee30551e441baa0c19c936f58a704a215e523c88e99bdec6a4f281fc9bf8be</t>
+          <t>c3107466a7804aae1e8b6cdbc47e767cbe96c23cba16058d4c3938feb836643d</t>
         </is>
       </c>
     </row>
@@ -1581,11 +1581,11 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>84804</v>
+        <v>81872</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>e76ef7bdd739d477778ddbb6fc7041afcc9fc3d9b292da5b92d1bd580c195934</t>
+          <t>67662b2a2c84f2221c902cb6ff557697bd92f9a4e9292f4e526e404b56e9381d</t>
         </is>
       </c>
     </row>
@@ -1596,11 +1596,11 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1186676</v>
+        <v>1212914</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>e5e1d869d315617342e7703e07263104717240eefe21046d9d6eaee2da0a0cac</t>
+          <t>5fe09b6465bae0438cfb3a37de8a3b0722a90a4cf39cd9831c4f2946268580e5</t>
         </is>
       </c>
     </row>
@@ -1615,7 +1615,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>49e7849bed2cbf5a3af29f9bfa72488baeb1f04a062c690e04d1a806be450f8c</t>
+          <t>9c9d63342d1e6a526c5a27ca5fcc723e27430611f430bc4c47a67dd320b1dd5b</t>
         </is>
       </c>
     </row>
@@ -1645,7 +1645,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>9c9db61371e8dadf062ac4589057466d04d3164a6219d6ae0526685644ae2279</t>
+          <t>7bce4f67c9b29ba8abbeceea7fc611f2094ab9ebb5b9b2c1b25c515e33b723da</t>
         </is>
       </c>
     </row>
@@ -1675,7 +1675,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>8967eaf6d8533c8a760b891ff04aa2f0a23251f9bbfb462bb6fddbf45c30a018</t>
+          <t>3bfb1f572bcf662377c32482f0bab4ba428bdbae51502048b97ff6b08cd91c9f</t>
         </is>
       </c>
     </row>
@@ -1705,7 +1705,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>f8fdc6177a692a4ce6161c531314929cf6554203d8a30d815f015e6ec4eea8cd</t>
+          <t>0fb8eba5dbe551df360f4f45870b289b41a6f6994b820a20d334b765855f5b52</t>
         </is>
       </c>
     </row>
@@ -1791,11 +1791,11 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>75669</v>
+        <v>75667</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>bf0f605340ce0ce33a4bc9a3dd952bf55372ffa03a501a471da7472f9fe74554</t>
+          <t>ed1510aad08213357a1874fb81cc5ecda662864c09f76d83047777242ec818a7</t>
         </is>
       </c>
     </row>
@@ -2436,11 +2436,11 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>4352</v>
+        <v>6628</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>54eed66c77212702829f3d4bc85907babd66e415997082a0a86a8b49ea1b4556</t>
+          <t>f6245e6b95476622c5ccdbabdd9819e0c5c449e8e2f38797f396dba21861150d</t>
         </is>
       </c>
     </row>
@@ -2451,11 +2451,11 @@
         </is>
       </c>
       <c r="B88" t="n">
-        <v>5734</v>
+        <v>8012</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>5a460deb7c3336af77955fa2de04d3386bb208a978ec8998174b14ce2f505fa3</t>
+          <t>f40ae7e1aaa5addf16fa4e2c943f108e37c73eac6b029232ad8d7837ed525e12</t>
         </is>
       </c>
     </row>
@@ -2466,11 +2466,11 @@
         </is>
       </c>
       <c r="B89" t="n">
-        <v>8751</v>
+        <v>12046</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>4e274bbb6e5a161f0079a012dd37cdd2d20d7558f1b2e2ac004d56269c814ddd</t>
+          <t>0c06b097a5a76e224113b94f072e43ee163953ea90201f9c29dcc3711c93ff58</t>
         </is>
       </c>
     </row>
@@ -2481,11 +2481,11 @@
         </is>
       </c>
       <c r="B90" t="n">
-        <v>4974</v>
+        <v>4954</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>710460457bcba4163b5d64d66b94ca476495f41a95378efddd2581ffa32a0196</t>
+          <t>2c82c18cd5897448165a93ce87e3423feccbe35155e74cee4d89cb6c7ad667dc</t>
         </is>
       </c>
     </row>
@@ -2571,11 +2571,11 @@
         </is>
       </c>
       <c r="B96" t="n">
-        <v>10358</v>
+        <v>14709</v>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>a6ea3da8d8d0928abbf9557443849e45ce01a97f2d7df368fc8c8c5c3a548501</t>
+          <t>39ebf4d77c3e9e04c9a622a204f137ec2789aa8e9fed6d7ba857138eb0feb16b</t>
         </is>
       </c>
     </row>
@@ -2586,26 +2586,26 @@
         </is>
       </c>
       <c r="B97" t="n">
-        <v>30537</v>
+        <v>31653</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>600e9aefde2898da31fc87ba4ca5d2878324ba73ec76f2b6b0d4704887c36794</t>
+          <t>d60260e90fd48ffe9f5eb643639d0b94f863e9346dc922ec16b33499578dc930</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>outputs/publication/D5_PUBLICATION_READINESS_AUDIT_v1.1.md</t>
+          <t>outputs/publication/D5_PUBLICATION_READINESS_AUDIT_v1.2.md</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>7400</v>
+        <v>7623</v>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>3000fd27bd303e5413d1d7eb5b5d7a464ac2e416930890be51a8a1928182ab5f</t>
+          <t>17e87ac6ee94ae2295677edb510245c808ce812f503bf29c4995e47e5b95b924</t>
         </is>
       </c>
     </row>
@@ -2665,7 +2665,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>c3a6003ecea1362dab936bfbad45fc6ef37294636555b31a7aa505186cff8080</t>
+          <t>568846bf82c1a60ce496d7724149414ac469e6978464d9a284e5b7a4717ae6e0</t>
         </is>
       </c>
     </row>
@@ -2676,11 +2676,11 @@
         </is>
       </c>
       <c r="B103" t="n">
-        <v>10601</v>
+        <v>11724</v>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>8c27e8a3c215ea325839dc203b968a69582e270588e1d5bb0fca1759624c4210</t>
+          <t>6838f382cacb25c9f1c1eff8afaebee4dccb71642e079232bed30438496ca8ca</t>
         </is>
       </c>
     </row>
@@ -2695,7 +2695,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>7619005d9470f6485750c452ea79fcfbff717ebab60ac2fb072170b5be2dd583</t>
+          <t>1ace1bc7ebbe577865e112f1ffb4910fc9a384bcfe46e8ab2d1ff0beb8e5f746</t>
         </is>
       </c>
     </row>
@@ -2710,7 +2710,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>300a6cb9e7b6f8c6c8ef1f043ddea916673046772105d1209cb6d9b1dbcabf3c</t>
+          <t>43dc129f8d845916e79369d3dd5c07546c375da8a8b64127945fa9c6f2f9bd8d</t>
         </is>
       </c>
     </row>
@@ -2721,11 +2721,11 @@
         </is>
       </c>
       <c r="B106" t="n">
-        <v>1075</v>
+        <v>1058</v>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>51b1250c4db8d4e2fc5fa97b2ebe2da15e4e47b37d9de1f8097b4e24b148ad20</t>
+          <t>53e0d073ef332fc162b7db37c204f7e803ab19e193a8adce3354f8cb59ac06aa</t>
         </is>
       </c>
     </row>
@@ -2826,11 +2826,11 @@
         </is>
       </c>
       <c r="B113" t="n">
-        <v>3904525</v>
+        <v>3942265</v>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>555acc56c3cbff9e389ab77b43e570a75b916697e57efb691387db00be069c2e</t>
+          <t>be2dedbef7c560882c3cb5a89778b001e9428c2003f987ed1dfb20dd1a9da3b4</t>
         </is>
       </c>
     </row>
@@ -2841,11 +2841,11 @@
         </is>
       </c>
       <c r="B114" t="n">
-        <v>10252</v>
+        <v>10364</v>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>1bc7c85d339d3df9deb1c08eafe0aa8b0b9c7d5e81a30b9e41ef39cfa4dbbd45</t>
+          <t>159d6a0c126fa64bc59844f3deeb4494baab692d9a7d559f35cfa6ba94957c80</t>
         </is>
       </c>
     </row>
@@ -2901,11 +2901,11 @@
         </is>
       </c>
       <c r="B118" t="n">
-        <v>4620</v>
+        <v>4538</v>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>8eebf74993e5b086730cf83b7953f1ae363c9e94dc2eb38ec7d3475a28496094</t>
+          <t>3bab49b975e41041916bbf003bedcaf390c7752a5418272d83e265867375eafc</t>
         </is>
       </c>
     </row>
@@ -3010,7 +3010,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>87c9c02f45ee2222bed152e5932338f8c4970970af051579544d809c7118d5c8</t>
+          <t>1072270e8cf7d3efdddc267aa49b1cd19f52b934979bb7b55636ac06fd50eec8</t>
         </is>
       </c>
     </row>
@@ -3021,11 +3021,11 @@
         </is>
       </c>
       <c r="B126" t="n">
-        <v>5732</v>
+        <v>5736</v>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>b7d9a57e289f30d49b4a1d54acb47d2d49b883b3d55ea7113af8ec21f836baf1</t>
+          <t>c1f9a23a8393c682257095dfa31c53a07256a104a52ccf89d1b83140d1246590</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Harden D5 support migration audit
</commit_message>
<xml_diff>
--- a/Project 1 Data Quality Assessment/D5 Topological Role Consistency and Structural Representativeness/outputs/local/D5_audit_log.xlsx
+++ b/Project 1 Data Quality Assessment/D5 Topological Role Consistency and Structural Representativeness/outputs/local/D5_audit_log.xlsx
@@ -1134,7 +1134,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C135"/>
+  <dimension ref="A1:C174"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1157,2008 +1157,2593 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>outputs/D5_RELEASE_QA.json</t>
+          <t>outputs/audit/support_migration/01_monthly_regime_occupancy.csv</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>28550</v>
+        <v>924</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>83aa7ba54fb6d2e9499c22134ddc210a67a151f8526abb6304ba2c0c8f992802</t>
+          <t>5347d963da5444a0be5bea88b976dda6fe876d709e0fc1a28c87b2ba0295173a</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>outputs/figures/D5_figure_qa.json</t>
+          <t>outputs/audit/support_migration/01_monthly_regime_occupancy.parquet</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>4935</v>
+        <v>5140</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>6197278780f24a12047422d29727861d98c8487defc691e4a60bb3bb50cf9b5a</t>
+          <t>0340167605fa9c9d10475d50763f838a712497cca690444afb0bb71e226a2ffe</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>outputs/figures/FigD5_1_framework.pdf</t>
+          <t>outputs/audit/support_migration/01b_pre_post_regime_shift.csv</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>51075</v>
+        <v>466</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>a872e0785320e7e8f6b15fef7f2ab4d167635bf4c74ccdefaab449f03c4ad25d</t>
+          <t>2473e9ea06589bc98d62288ccf065ec7ca6029c6131a8c3abfc861bc5995ccb2</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>outputs/figures/FigD5_1_framework.png</t>
+          <t>outputs/audit/support_migration/01b_pre_post_regime_shift.parquet</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>401779</v>
+        <v>5720</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>347e59f63f0c1cdf329f7375c27f3516c79e5068b4ea597ee43af1aa7d6e8236</t>
+          <t>4caf10426c2e69948060978bca58a2e72b59fc3f7d6605af031f5058212cceca</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>outputs/figures/FigD5_1_framework.svg</t>
+          <t>outputs/audit/support_migration/02_template_occupancy_56.csv</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>44204</v>
+        <v>61443</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>412c49bfe1e3289c79ed9039c14e4b817fd6ecd6880c7adb400eb541d2aa2afe</t>
+          <t>fb197bde632972433adc93676c070d4cace136159060bfdfc84888b777498231</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>outputs/figures/FigD5_1_framework.tiff</t>
+          <t>outputs/audit/support_migration/02_template_occupancy_56.parquet</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>982482</v>
+        <v>59044</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>6c436b0badd0f3728278bf32e8e188eee38e9b0ab8122de2f6731b9e5f2a49de</t>
+          <t>9f198235c034d7b3eaa361a19c0520aabc2d03a65995a1eea7187608962c398b</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>outputs/figures/FigD5_2_spatiotemporal.pdf</t>
+          <t>outputs/audit/support_migration/03_L1_to_L2_blockers.csv</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>57597</v>
+        <v>19374</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>16fb7f73931ef0bcc5044c55147e22c1e5b4d9198fc0ceaabba68e1d8236dfb8</t>
+          <t>723ed00365f968c964394181c4855f3b1776c6e441050b32a67cfcd200946868</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>outputs/figures/FigD5_2_spatiotemporal.png</t>
+          <t>outputs/audit/support_migration/03_L1_to_L2_blockers.parquet</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>342819</v>
+        <v>57939</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>1a3693d32cb3698bf270272eaa1454fcb0cb327b09c0d4f07d2558e752bdc884</t>
+          <t>213d03732a77af47ec8b1ae4fa96b0a26c4eb0f63439a32c34ed7b6e7836eaf6</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>outputs/figures/FigD5_2_spatiotemporal.svg</t>
+          <t>outputs/audit/support_migration/04_L2_to_L3_blockers.csv</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>59173</v>
+        <v>48740</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>7aea48aa61203adb09fa646cd3935f09c2a544db6d6ce16b1d5c15022f637b76</t>
+          <t>48d1d700d0905237c97f535df63247c1650c0f8f22c47b74f309b2804b2d93ae</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>outputs/figures/FigD5_2_spatiotemporal.tiff</t>
+          <t>outputs/audit/support_migration/04_L2_to_L3_blockers.parquet</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>8197140</v>
+        <v>63522</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>453f55b4cbe5768323d20ed751a9ca0224df7ac78039010c8de90c4f107112ec</t>
+          <t>d84777bacf5580e70805956913b264ba4df5c8e6423670e2234d60f3043cd7e8</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>outputs/figures/FigD5_3_evidence.pdf</t>
+          <t>outputs/audit/support_migration/05_coverage_loss_attribution.csv</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>54259</v>
+        <v>469</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>0360a1c00cfe7e0c80f9ab49d0e587dffcf9a69973e58c8f410d2fae2747272e</t>
+          <t>714c034d5f1beb94038c13ab34be16befe802dd3afc986680e7750f77ed1a9f1</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>outputs/figures/FigD5_3_evidence.png</t>
+          <t>outputs/audit/support_migration/05_coverage_loss_attribution.parquet</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>590613</v>
+        <v>6069</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>579af665f82a2b29865d392e3d74537346efbe4f2fdc7c0125cc31fd30404314</t>
+          <t>a3df615816060627339ba74926e06f98374c201a51f6e0600d2b68ee78439709</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>outputs/figures/FigD5_3_evidence.svg</t>
+          <t>outputs/audit/support_migration/06_counterfactual_coverage.csv</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>64408</v>
+        <v>430</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>be3822405e2c14214629ff549e51121033850093cc454593ec5fad7937851189</t>
+          <t>2931a2814daa7dbb3e3554bf71317442963bf75ac21e98643e9da7258283ddac</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>outputs/figures/FigD5_3_evidence.tiff</t>
+          <t>outputs/audit/support_migration/06_counterfactual_coverage.parquet</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1246956</v>
+        <v>4093</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ce6ddfc9adca0b09fadff514018446089063d21627cf2f4a86f76566e01ea7dd</t>
+          <t>1b404b74d113f445ba704c0b0a7b9fca7bbde2a8376b4067fd91159f680b63b7</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>outputs/figures/FigD5_4_validation.pdf</t>
+          <t>outputs/audit/support_migration/07_reference_horizon_sensitivity.csv</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>48538</v>
+        <v>1502</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>c08f738254549d88fda6d7ddf70b6e6f79fa7fd773fdf93e761fa033708d8b16</t>
+          <t>6ea9bff9843486b209e330ff6180565947484dcb47947aa72f505eb57b1ee8d8</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>outputs/figures/FigD5_4_validation.png</t>
+          <t>outputs/audit/support_migration/07_reference_horizon_sensitivity.parquet</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>539959</v>
+        <v>6627</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>3783592511e27dd37446d891c95d88e70ad444942531f54820f8dbfa438f0a12</t>
+          <t>11a45e83adbb3d9fb6ee071280cb1552e8f0d38a5b15b1017d2c3f00403f60e8</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>outputs/figures/FigD5_4_validation.svg</t>
+          <t>outputs/audit/support_migration/08_monthly_report_eligibility.csv</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>46632</v>
+        <v>726</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>fef0c6e7297f56553b0acb7c2441dc67bb49cb3d5d526d5bd018a27697bf51a6</t>
+          <t>8b1b64145508b6c569118e9f6167a99a575c276bac01044a54f70ff18af29585</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>outputs/figures/FigD5_4_validation.tiff</t>
+          <t>outputs/audit/support_migration/08_monthly_report_eligibility.parquet</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1418876</v>
+        <v>4540</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>d42e75853c77121516bbc34a59c005fdee056bff211907a1269b4708db19a0ec</t>
+          <t>d34de153122c0c474939f269271a0265a386f7b3b592eb3a6cd6a5a3ba45207a</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>outputs/figures/FigD5_5_governance.pdf</t>
+          <t>outputs/audit/support_migration/D5_support_migration_audit.xlsx</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>62555</v>
+        <v>67591</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>bc4a257d4b3669abeb3872eadb78119e9f2a2d2ff426028040735e84c8587139</t>
+          <t>f47c074542a0d05e3049c2655702e94f4ac32806a15a452530594698db82af7f</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>outputs/figures/FigD5_5_governance.png</t>
+          <t>outputs/audit/support_migration/D5_SUPPORT_MIGRATION_AUDIT_REPORT.md</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>484038</v>
+        <v>4237</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>f931dad797efa29713ce271068677d91cda7a985b123f9539c886bb6c3ba7dc2</t>
+          <t>b91c1ad0a8b2c7cbfa9a8b1a5fbe498e8d240480bc212613288826e9862fa89d</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>outputs/figures/FigD5_5_governance.svg</t>
+          <t>outputs/audit/support_migration/D5_support_migration_manifest.json</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>56460</v>
+        <v>9662</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>a9cdb0c0a34753e20cc9946ae5b75df42741d4118a2aad58006770e690fe1624</t>
+          <t>6f9c815df1932a4107adc4a02e153c2f547bb8afe0d0891b722b7e76966a6642</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>outputs/figures/FigD5_5_governance.tiff</t>
+          <t>outputs/D5_RELEASE_QA.json</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1182478</v>
+        <v>36870</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>c928a1e6e2a7517e6002c22db7c7a1f829c86a6555c6d34b2a44c3dd8ee11c82</t>
+          <t>ecdc7d0bc38ff52ecb173e583ec8d0dd64bb20cc9124d779c742d4f3010c192d</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>outputs/figures/FigD5_6_validation_coverage.pdf</t>
+          <t>outputs/figures/D5_figure_qa.json</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>54719</v>
+        <v>7580</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>bd8b424c251d78568c23fd1dee1f0804d3cd0966daca1fbd5fdbf540df016cbb</t>
+          <t>1d0c4e815827302ce0f19cc80dea5ff1028c03f19cf67f5676ad21c41e8290f3</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>outputs/figures/FigD5_6_validation_coverage.png</t>
+          <t>outputs/figures/FigD5_1_framework.pdf</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>656187</v>
+        <v>51250</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>a5d0f89175f27a60c6eeca284615c672b5fa47f41fbbecf3c25d67ee17718553</t>
+          <t>700bb88943fb9810b204d6823f01eb5cf3c1bde5c143a6422b752bbd8fb80967</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>outputs/figures/FigD5_6_validation_coverage.svg</t>
+          <t>outputs/figures/FigD5_1_framework.png</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>69085</v>
+        <v>382812</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>5b19aa268856963bd00229b76088adc9675c3a3436dcb4085c05db3c61cb0953</t>
+          <t>0b2446b6d9140788a1bcf9f67c0bc6935e14040a400b296a583c6db98855ff9e</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>outputs/figures/FigD5_6_validation_coverage.tiff</t>
+          <t>outputs/figures/FigD5_1_framework.svg</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>1389316</v>
+        <v>41052</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>767b8e085c5fa28f4211ab49ed95097a666f52963742ae45fec71e2bfe93b160</t>
+          <t>81fa39166769bfbd5200878ccf5df9f293dfe03cf216bc6065b9d7375d93a5f2</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>outputs/figures/FigD5_7_D4_D5_complementarity.pdf</t>
+          <t>outputs/figures/FigD5_1_framework.tiff</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>58200</v>
+        <v>1035836</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>8a1bd5a137ec759b81994ef7e9551cf10bd2c81477915a64adc2ca1831f50ff3</t>
+          <t>c0d57c017959f234eab3f20a81818ec333a340f21a04f90934ec079b5b9809ff</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>outputs/figures/FigD5_7_D4_D5_complementarity.png</t>
+          <t>outputs/figures/FigD5_2_spatiotemporal.pdf</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>590625</v>
+        <v>69945</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>c3107466a7804aae1e8b6cdbc47e767cbe96c23cba16058d4c3938feb836643d</t>
+          <t>78e495172970e229f4e43a04eaf13b5c4f38ed8657764e51181461d26b5b7579</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>outputs/figures/FigD5_7_D4_D5_complementarity.svg</t>
+          <t>outputs/figures/FigD5_2_spatiotemporal.png</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>81872</v>
+        <v>644906</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>67662b2a2c84f2221c902cb6ff557697bd92f9a4e9292f4e526e404b56e9381d</t>
+          <t>b4c93b8bcfd46f52d38c85251f2ff4e9e3451f864aa1893fa31200d3b0f46bb5</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>outputs/figures/FigD5_7_D4_D5_complementarity.tiff</t>
+          <t>outputs/figures/FigD5_2_spatiotemporal.svg</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1212914</v>
+        <v>95904</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>5fe09b6465bae0438cfb3a37de8a3b0722a90a4cf39cd9831c4f2946268580e5</t>
+          <t>61db4a191706f4995593331e103da9a66214d73d1e48f81b8507f8c2419ea92a</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>outputs/figures/FigD5_8_dimension_availability_sensitivity.pdf</t>
+          <t>outputs/figures/FigD5_2_spatiotemporal.tiff</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>53301</v>
+        <v>6443510</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>9c9d63342d1e6a526c5a27ca5fcc723e27430611f430bc4c47a67dd320b1dd5b</t>
+          <t>f52d34f934898c030d31ded59048cd5a1351565279c7a3eac1dedc0fee2dc829</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>outputs/figures/FigD5_8_dimension_availability_sensitivity.png</t>
+          <t>outputs/figures/FigD5_3_evidence.pdf</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>535313</v>
+        <v>56040</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>25eed423cc1a6f55d00a2658d7ce4a3fd7a3e60bad1fdf6a6f6f4ff5cc3d51cb</t>
+          <t>076cda73773cad1ae77847209850e5dab91c8ce8dfc345e2365cbb3a41eb5675</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>outputs/figures/FigD5_8_dimension_availability_sensitivity.svg</t>
+          <t>outputs/figures/FigD5_3_evidence.png</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>69730</v>
+        <v>718126</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>7bce4f67c9b29ba8abbeceea7fc611f2094ab9ebb5b9b2c1b25c515e33b723da</t>
+          <t>47ceafcc44de75dfe3b6d904b6eac897c8a3a43e4e3d773aa9fda4bb8c592ceb</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>outputs/figures/FigD5_8_dimension_availability_sensitivity.tiff</t>
+          <t>outputs/figures/FigD5_3_evidence.svg</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>1406590</v>
+        <v>105761</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>5e3895e9fe1ed2a5ad7e18aba0096ca11933e581e01f1cfc3cd65a08927cc045</t>
+          <t>c280a65995a28d1c23a954cc0a69136940c192de67dfa7a81a7bfaa98563c31f</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>outputs/figures/FigD5_9_target_support_robustness.pdf</t>
+          <t>outputs/figures/FigD5_3_evidence.tiff</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>48906</v>
+        <v>1825322</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>3bfb1f572bcf662377c32482f0bab4ba428bdbae51502048b97ff6b08cd91c9f</t>
+          <t>7c4728a4cbe297d88840a97c3843091026e6d3a90f305932b70a560928238084</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>outputs/figures/FigD5_9_target_support_robustness.png</t>
+          <t>outputs/figures/FigD5_4_validation.pdf</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>406917</v>
+        <v>42966</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>fd0415d6e3ed87344cc5140186fd9b86626bfd1225dfd72662dae3042f1f5360</t>
+          <t>51a8b842ce5478a5017e32b80840fa9cc9d619a6306429cd6da4c2f38eee8048</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>outputs/figures/FigD5_9_target_support_robustness.svg</t>
+          <t>outputs/figures/FigD5_4_validation.png</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>35150</v>
+        <v>531658</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>0fb8eba5dbe551df360f4f45870b289b41a6f6994b820a20d334b765855f5b52</t>
+          <t>4dabbd36451b1fe017eda7bd18c5639d13c38b776456513befb056d730c546c5</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>outputs/figures/FigD5_9_target_support_robustness.tiff</t>
+          <t>outputs/figures/FigD5_4_validation.svg</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>1040878</v>
+        <v>37071</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>88af281d37f8851618be048e49a8313a4a1a8a3a1e1d3f452a9b911daca6168d</t>
+          <t>5cfbf6dc9d2a80409bbcf288da522083dec40e53fc51193e7412c4cc00fc5e5a</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>outputs/figures/figure_bundle_audit.json</t>
+          <t>outputs/figures/FigD5_4_validation.tiff</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>2409</v>
+        <v>1226424</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>da3ebd141c082e91a1745abc60394a9bc5c09de0cd31ad6297aa5cafc4d49756</t>
+          <t>29ae2daaa9e73c6936fc202a572a0b8dc48b0660ca2aaaf676c347667804ae53</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>outputs/local/D5_ablation_redundancy.xlsx</t>
+          <t>outputs/figures/FigD5_5_governance.pdf</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>9984</v>
+        <v>56106</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>f0feb1f3c9868bf39b167645436a3c13adea0cb6253ce840188905750b8c2157</t>
+          <t>0f8d01e72727cc30111b1bc34cfd648075d07dbbe40553905d20ae8c2fa57cf1</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>outputs/local/D5_admission_decision.json</t>
+          <t>outputs/figures/FigD5_5_governance.png</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>588</v>
+        <v>435410</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>a9c40d2d57897245afa23202d8e7ba49245ff63b19b9427ab86d12003a4c1583</t>
+          <t>a0f780e4b66a562d250a8c8649b40d74cc722a0c43fe1a382765afdcea2c6e70</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>outputs/local/D5_admission_decision.xlsx</t>
+          <t>outputs/figures/FigD5_5_governance.svg</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>6135</v>
+        <v>48485</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>96cce073f38f1f8e9d436722f18513ea84f6acf4ba33920ca07d1185db5767dd</t>
+          <t>cb33105e67e0b4832b4e728ee303bdc081e6e0dfdaa18c7ee45db094003c6e6f</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>outputs/local/D5_audit_log.xlsx</t>
+          <t>outputs/figures/FigD5_5_governance.tiff</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>75667</v>
+        <v>1078506</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>ed1510aad08213357a1874fb81cc5ecda662864c09f76d83047777242ec818a7</t>
+          <t>7c17e2721f228a98f24acc27dd5d2623e1b127900a39f9b7b2054ab70e08fc44</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>outputs/local/D5_case_study_exports.xlsx</t>
+          <t>outputs/figures/FigD5_6_validation_coverage.pdf</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>44198</v>
+        <v>50513</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>060027cb3475620e45c16a5aed24ec4f94b00c01a7a3ba027a188963d7682dbc</t>
+          <t>fae69822c06d7028036c0c4a88a870226921ca8b43c71d52f7724fd5518d7ee6</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>outputs/local/D5_edge_profile_summary.xlsx</t>
+          <t>outputs/figures/FigD5_6_validation_coverage.png</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>26857</v>
+        <v>638938</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>5b3bd2c7f60bb706732433cc146f79297976ea8f202150b40c281c932b3a6329</t>
+          <t>3142461a1958b6109fa039e5a77a089ee36f928bd138f9bb12a01f3cad740c63</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>outputs/local/D5_event_windows.parquet</t>
+          <t>outputs/figures/FigD5_6_validation_coverage.svg</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>80614</v>
+        <v>58383</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2874ab1d42be1723d6baabd3bd81b768d9f4b3fcf5459712e226f029f25a24fd</t>
+          <t>7d263bc9dbe719410f6fe02ff2ff2c86a8d61133ea85131a4f3031aac9c4b5f2</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>outputs/local/D5_event_windows.xlsx</t>
+          <t>outputs/figures/FigD5_6_validation_coverage.tiff</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>140097</v>
+        <v>1346336</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>97f101d88e4b67e9376735a772083ed8f1403eb700de6666b4a51314b7bc3dae</t>
+          <t>f670f0c97d0cfec2fbcfcb834f5a843adb273c98dcce661631166ec9e6f0167b</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>outputs/local/D5_gate_interface.parquet</t>
+          <t>outputs/figures/FigD5_7_D4_D5_complementarity.pdf</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>796803</v>
+        <v>59590</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>22b640fa64ff95f0677bdcafea1517c192dd506fc11559efc53db49916918e0e</t>
+          <t>1a86275a0c8388633a626f5b3c058c39ceb6f7701f87318bbba64882b5fe2332</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>outputs/local/D5_gate_interface.schema.json</t>
+          <t>outputs/figures/FigD5_7_D4_D5_complementarity.png</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>1128</v>
+        <v>941070</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>619b0d9ef22475a5de39a752b479540987d05f9cb5d649e2f7bece38005622f3</t>
+          <t>390c439b2d1f72e3570a3b9fed2cf9e086a2b7c2dd574593978c7ac49fae1c50</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>outputs/local/D5_gate_interface.xlsx</t>
+          <t>outputs/figures/FigD5_7_D4_D5_complementarity.svg</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>5209423</v>
+        <v>201110</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>cc6458fcb96aa750a01b53bb7acfaceae4f832b53e68bd1840f57a8ee787b22c</t>
+          <t>49011a417bc95f4bd4a66fdac07618609b4c32e5417c26ea45ff6d6cf13df21b</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>outputs/local/D5_main_scores_hourly.parquet</t>
+          <t>outputs/figures/FigD5_7_D4_D5_complementarity.tiff</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>7340495</v>
+        <v>3106950</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>64274562d7139d510dd3780dbd67bd2c2c5913908dbbec8ac7d4bcceb0418cd1</t>
+          <t>5db501d151d430f33be6dcf747f3c339ec0fb67fdd29f5bc1ba969f237dec583</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>outputs/local/D5_main_scores_hourly.xlsx</t>
+          <t>outputs/figures/FigD5_8_dimension_availability_sensitivity.pdf</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>45272583</v>
+        <v>48207</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>2ae0e3dcb195bddabcb98ac87479345348da28818c565a978c56f75ff0ee19c9</t>
+          <t>ec13a44b05b79bf3ba09bc2ca014db34668406e4f23edcdcf0da2d7d4da81bc0</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>outputs/local/D5_mapping_params.xlsx</t>
+          <t>outputs/figures/FigD5_8_dimension_availability_sensitivity.png</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>20237</v>
+        <v>507591</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>30ffe256d465c57c614fcab9fa40d92fcd68a7c1f5fc78cbd8e0e0d00779b6a6</t>
+          <t>d123ff696b47fc1ec14a9b2face98833eb5e69460a4277b9703974902284d091</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>outputs/local/D5_multiscale_aggregates.xlsx</t>
+          <t>outputs/figures/FigD5_8_dimension_availability_sensitivity.svg</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>1060062</v>
+        <v>58107</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>96da07e011eecb169c1880e11e5c8656c9aa16a62434b3ad540a8b9a658a5da0</t>
+          <t>d30a40b1fc0862d48826e5be2352894c388234d470613d7609060b232a48b4d3</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>outputs/local/D5_reference_window_library.parquet</t>
+          <t>outputs/figures/FigD5_8_dimension_availability_sensitivity.tiff</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>62947</v>
+        <v>1322456</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>b84bd8208e2e533e83c722868f022eaf87e07991f184e6d59e9411909e5360bc</t>
+          <t>45c025977c8dda152a05ab27d993512b7982c7f8a09fcd6cefea183a7178ed2a</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>outputs/local/D5_reference_window_library.xlsx</t>
+          <t>outputs/figures/FigD5_9_target_support_robustness.pdf</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>228952</v>
+        <v>47131</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>12bb084003accca5fd0e85f42191286a56a27c7016b617296cde45ff4004edf1</t>
+          <t>2e582cbfa3a4107275a4633b77b34688efc1ddab583723b55fc44b0022732506</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>outputs/local/D5_regime_state.parquet</t>
+          <t>outputs/figures/FigD5_9_target_support_robustness.png</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>3658910</v>
+        <v>428997</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>622dd0f5ed1473ae5de464e4207e51ff9470de209cadcee9b30cbac92f9392e8</t>
+          <t>fddb68afe2f9776046e153e66f44530295cc60cb576349dd370c4f51e0492d5f</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>outputs/local/D5_regime_state.xlsx</t>
+          <t>outputs/figures/FigD5_9_target_support_robustness.svg</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>45834835</v>
+        <v>47007</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>427fe81df8b7861210e267f694058376a754fa724e0bbafe1b07208e32787485</t>
+          <t>33bd39117fca81cb32722cefdd673e69ce1f32c56e66ed02093b6e649b3a4ca0</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>outputs/local/D5_report_interface.parquet</t>
+          <t>outputs/figures/FigD5_9_target_support_robustness.tiff</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>1171194</v>
+        <v>1162650</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>f057e0a8037282fb43a71a94d7043c7bd3de2b4c8fa9865365bcf0427195dbda</t>
+          <t>106f932ac54a22077b2b2fdef769d91f4348d62cfa9189d003833abdee64bef1</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>outputs/local/D5_report_interface.schema.json</t>
+          <t>outputs/figures/figure_bundle_audit.json</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>853</v>
+        <v>2409</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>c740ff5a12c99a1a761c5f2ab45d12f5174aaac3b2201e58e6d67a1a8c87c06e</t>
+          <t>da3ebd141c082e91a1745abc60394a9bc5c09de0cd31ad6297aa5cafc4d49756</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>outputs/local/D5_report_interface.xlsx</t>
+          <t>outputs/figures/supplementary/support_migration/FigD5_S1_monthly_regime_occupancy_migration.pdf</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>11410677</v>
+        <v>29778</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>f9040450b3fb8204f2fea44f92c003d1cdc2acf900a29715ee732a8b9b450aae</t>
+          <t>3b48fa368ee8089ca9a664d9373ad8a8f295d3cffe40c10cc393b643630a968c</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>outputs/local/D5_sensor_influence.parquet</t>
+          <t>outputs/figures/supplementary/support_migration/FigD5_S1_monthly_regime_occupancy_migration.png</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>6011187</v>
+        <v>195025</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>a9270494760fcb4ae501abcf54c50e813ca74d6306d7fbca94d7ef1a1d1730a2</t>
+          <t>5e1f70b1e62d83b95e3d139cd5ad98211537b31b82ca8e40ec2e9981dc9bc71d</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>outputs/local/D5_sensor_influence.xlsx</t>
+          <t>outputs/figures/supplementary/support_migration/FigD5_S1_monthly_regime_occupancy_migration.svg</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>16403976</v>
+        <v>20776</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>338920c1db9c7b1bc500fa43d92f02f6165187545a79f696771287bfd877a9a0</t>
+          <t>1ccdbda0b661c80755bb837e8db1962f64bd3813d8fb959b128fe7778ecb1bf0</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>outputs/local/D5_sensor_profile_summary.xlsx</t>
+          <t>outputs/figures/supplementary/support_migration/FigD5_S1_monthly_regime_occupancy_migration.tiff</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>7442</v>
+        <v>1043412</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>aef38bd66378a9ae3b2c76a848f1ef4d51d504616c435440e45f99eadf9fb5a9</t>
+          <t>e958b1233a6d3bd2be00cca100cd572bc83415f7afd76b4bff099eeaf42496e8</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>outputs/local/D5_spatial_evidence.parquet</t>
+          <t>outputs/figures/supplementary/support_migration/FigD5_S2_sensor_regime_maturity_map.pdf</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>6146048</v>
+        <v>38804</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>4edb2bd1af0cbdac8fc61382508099137349f67f6ce70da4ee1831848bfe3733</t>
+          <t>2ddc6819a7fb31605ddc2e10b58788d1270f979388ae4fd8d99c39e29dda87e8</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>outputs/local/D5_spatial_evidence.xlsx</t>
+          <t>outputs/figures/supplementary/support_migration/FigD5_S2_sensor_regime_maturity_map.png</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>15958642</v>
+        <v>275575</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>6e2a433bcdb115b841f269c5eb5184623502c7221234da51b8ade0377c120327</t>
+          <t>40458ba4446cf8d8313396c0930a4b00ccf884a0f9cbefa0d34fccfc061bf48d</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>outputs/local/D5_spatial_templates.template_bundle.json</t>
+          <t>outputs/figures/supplementary/support_migration/FigD5_S2_sensor_regime_maturity_map.svg</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>542571</v>
+        <v>39126</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>704238fcb5551593e569bdb3e015f04cb710815fdeccbb8aa28ba9a0c7e59ace</t>
+          <t>a7bf01c9476fc145994131e4745f3a43b3497fd8d2841e3800cf2986af0c6e4d</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>outputs/local/D5_spatial_templates.xlsx</t>
+          <t>outputs/figures/supplementary/support_migration/FigD5_S2_sensor_regime_maturity_map.tiff</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>190694</v>
+        <v>1392684</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>6fc3291e19dd0663ccd33db897edbf39e67f54e7db7b1fa8de0648d06d82c6bc</t>
+          <t>5c6f3c5d7eb36085b5d5f21fe2169bf3e66fada3864a0701b5ae89d6671dd94f</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>outputs/local/D5_support_assessment.parquet</t>
+          <t>outputs/figures/supplementary/support_migration/FigD5_S3_L1_blocker_matrix.pdf</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>52815</v>
+        <v>40167</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>00d3ed69dc3899db48c841bb56c6664bc1832e365fd5fa5c13130b6d231e5750</t>
+          <t>acf60514c88051c998ba51e7d798a1f66a61d681e08a7661f34ee6901ee4385b</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>outputs/local/D5_support_assessment.xlsx</t>
+          <t>outputs/figures/supplementary/support_migration/FigD5_S3_L1_blocker_matrix.png</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>28036</v>
+        <v>348233</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>34df65d8e4329d166c69a9bc505bb97a8397e537f323c5be392fba093827dd98</t>
+          <t>2345fbdefea8145e9381062a108efb0768849f9aa14039e98c154e9022bad8d9</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>outputs/local/D5_topology_drift_alerts.parquet</t>
+          <t>outputs/figures/supplementary/support_migration/FigD5_S3_L1_blocker_matrix.svg</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>10824</v>
+        <v>33759</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>59d05a6c138fc18e295611bb0e39f469c07f6a25522ed809ea4f76ca018a908a</t>
+          <t>e2e06ba5c1c261b5fe42909001284448ecbd85ba865001d792118cdcbec6360f</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>outputs/local/D5_topology_drift_alerts.xlsx</t>
+          <t>outputs/figures/supplementary/support_migration/FigD5_S3_L1_blocker_matrix.tiff</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>9965</v>
+        <v>1567634</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>7262caaddcf1713a512e6dd52157f3f0e4bee9ae2642dcaf63eed60ff9ce9a87</t>
+          <t>d9de222dae61272c2f284bc66286dee13048aeed54acd811b89d51a206535642</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>outputs/local/D5_topology_evidence.yaml</t>
+          <t>outputs/figures/supplementary/support_migration/FigD5_S4_counterfactual_coverage_recovery.pdf</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>2342</v>
+        <v>37933</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>50abd276a9e6bbf26acb9a22d3a796ca63423d363a036422dc57c6bdfeb71920</t>
+          <t>5585aaa9b1c03df4ef784a49a7b966e62edb852cdd5764c9380af9dc012aef74</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>outputs/local/D5_topology_registry.json</t>
+          <t>outputs/figures/supplementary/support_migration/FigD5_S4_counterfactual_coverage_recovery.png</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>14821</v>
+        <v>226217</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>6efbf6722e2caecabf2d9999637d48bbb7c4d630dc3e9354982ed89d750965bc</t>
+          <t>c5f9e1f2e5bc01173f14c8a5b63a2cc48b13dbf3daf0f9f2bb02ea1b581dfb82</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>outputs/local/D5_topology_registry.schema.json</t>
+          <t>outputs/figures/supplementary/support_migration/FigD5_S4_counterfactual_coverage_recovery.svg</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>1301</v>
+        <v>12664</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>0f4c6e9e6d510996d1435efd1810b4a1eaca35a989b7f3d78187e29f8ce9584e</t>
+          <t>50164792453a9582ca727bc14f874a0287350f4f9c727263ffd187b87fe7957f</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>outputs/local/D5_topology_registry.xlsx</t>
+          <t>outputs/figures/supplementary/support_migration/FigD5_S4_counterfactual_coverage_recovery.tiff</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>11679</v>
+        <v>508582</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>7aa5db4087c2346acc99d827f7c3a0bd49ce90540fb2ec8f56664c82b14e36ff</t>
+          <t>a0355132dc0114e57ce52efb1cce2c7a21a43dd52dd6d9f84adedb3051c3ba2b</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>outputs/local/D5_topology_registry.yaml</t>
+          <t>outputs/local/D5_ablation_redundancy.xlsx</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>2838</v>
+        <v>9984</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>46e191549a0c768ee947bff4d98f26f38a93ecbce380ab4ff8114d2885dd29f9</t>
+          <t>f0feb1f3c9868bf39b167645436a3c13adea0cb6253ce840188905750b8c2157</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>outputs/local/D5_validation_results.xlsx</t>
+          <t>outputs/local/D5_admission_decision.json</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>64326</v>
+        <v>588</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>b4a0f5586b1108b945dba84b87a47a7f387c11fa182de0c506977f3c9870efff</t>
+          <t>a9c40d2d57897245afa23202d8e7ba49245ff63b19b9427ab86d12003a4c1583</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>outputs/local/D5_zone_consensus.parquet</t>
+          <t>outputs/local/D5_admission_decision.xlsx</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>1618880</v>
+        <v>6135</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>0cb43651f4dc8c4a7f378cfe3be964a688e7df7a2ff45052f649259b415cdb8c</t>
+          <t>96cce073f38f1f8e9d436722f18513ea84f6acf4ba33920ca07d1185db5767dd</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>outputs/local/D5_zone_consensus.xlsx</t>
+          <t>outputs/local/D5_audit_log.xlsx</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>7277838</v>
+        <v>78456</v>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>f43c5554c5a0c9f3e50e38f51bc0db270a9c819c3a00a9f3dc23ae658b7e7149</t>
+          <t>1be6c6483c163b412ced24fd772f84f673d2c14aecf3907d4f9b03ef516e9679</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>outputs/plot_data/D5_plot_data.csv</t>
+          <t>outputs/local/D5_case_study_exports.xlsx</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>18506701</v>
+        <v>44198</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>f074d7394f60df5f9b874734fe644757863bf44e876dd97303344227afe065c3</t>
+          <t>060027cb3475620e45c16a5aed24ec4f94b00c01a7a3ba027a188963d7682dbc</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>outputs/plot_data/D5_plot_data.parquet</t>
+          <t>outputs/local/D5_edge_profile_summary.xlsx</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>744459</v>
+        <v>26857</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>3236229f520cfa38329877aa013a7233229a77567e32c95b37a87d5fe94a5dd8</t>
+          <t>5b3bd2c7f60bb706732433cc146f79297976ea8f202150b40c281c932b3a6329</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>outputs/plot_data/D5_plot_data_manifest.json</t>
+          <t>outputs/local/D5_event_windows.parquet</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>519</v>
+        <v>80614</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>27ae5a05d462aab27e6a6359daaf99d931840e8b58d462da108ff3ca12dfc1ae</t>
+          <t>2874ab1d42be1723d6baabd3bd81b768d9f4b3fcf5459712e226f029f25a24fd</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>outputs/publication/D5_coverage_strata.parquet</t>
+          <t>outputs/local/D5_event_windows.xlsx</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>5837</v>
+        <v>140097</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>f4da589996c29b4e710131be262c3efdaa0fb822e051293f1310365aaf0e7b75</t>
+          <t>97f101d88e4b67e9376735a772083ed8f1403eb700de6666b4a51314b7bc3dae</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>outputs/publication/D5_coverage_summary.parquet</t>
+          <t>outputs/local/D5_gate_interface.parquet</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>2879</v>
+        <v>796803</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>54201e6be7009f8ed97eb53e8abd9d8d33766757486839e1d1650d09bf1718c6</t>
+          <t>22b640fa64ff95f0677bdcafea1517c192dd506fc11559efc53db49916918e0e</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>outputs/publication/D5_d4_d5_composite.parquet</t>
+          <t>outputs/local/D5_gate_interface.schema.json</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>6628</v>
+        <v>1128</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>f6245e6b95476622c5ccdbabdd9819e0c5c449e8e2f38797f396dba21861150d</t>
+          <t>619b0d9ef22475a5de39a752b479540987d05f9cb5d649e2f7bece38005622f3</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>outputs/publication/D5_d4_d5_dependence.parquet</t>
+          <t>outputs/local/D5_gate_interface.xlsx</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>8012</v>
+        <v>5209423</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>f40ae7e1aaa5addf16fa4e2c943f108e37c73eac6b029232ad8d7837ed525e12</t>
+          <t>cc6458fcb96aa750a01b53bb7acfaceae4f832b53e68bd1840f57a8ee787b22c</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>outputs/publication/D5_d4_d5_stratified_rho.parquet</t>
+          <t>outputs/local/D5_main_scores_hourly.parquet</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>12046</v>
+        <v>7340495</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>0c06b097a5a76e224113b94f072e43ee163953ea90201f9c29dcc3711c93ff58</t>
+          <t>64274562d7139d510dd3780dbd67bd2c2c5913908dbbec8ac7d4bcceb0418cd1</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>outputs/publication/D5_decision_register.parquet</t>
+          <t>outputs/local/D5_main_scores_hourly.xlsx</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>4954</v>
+        <v>45272583</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>2c82c18cd5897448165a93ce87e3423feccbe35155e74cee4d89cb6c7ad667dc</t>
+          <t>2ae0e3dcb195bddabcb98ac87479345348da28818c565a978c56f75ff0ee19c9</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>outputs/publication/D5_dimension_availability.parquet</t>
+          <t>outputs/local/D5_mapping_params.xlsx</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>12550</v>
+        <v>20237</v>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>f34750499b681fb5eefe3f811fbbec3a4d0570f45ca71a850a191b4a67c93680</t>
+          <t>30ffe256d465c57c614fcab9fa40d92fcd68a7c1f5fc78cbd8e0e0d00779b6a6</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>outputs/publication/D5_localization.parquet</t>
+          <t>outputs/local/D5_multiscale_aggregates.xlsx</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>6980</v>
+        <v>1060062</v>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>e63682e2c8a0ebeb772d9d0eae21b4be654b370f853eb939376249c595ddfcff</t>
+          <t>96da07e011eecb169c1880e11e5c8656c9aa16a62434b3ad540a8b9a658a5da0</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>outputs/publication/D5_monthly_coverage.parquet</t>
+          <t>outputs/local/D5_reference_window_library.parquet</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>6919</v>
+        <v>62947</v>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>51e4fd571650b85d5e4d8c2aab7c0ca543cb81aff01517a7efacc70c08bea506</t>
+          <t>b84bd8208e2e533e83c722868f022eaf87e07991f184e6d59e9411909e5360bc</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>outputs/publication/D5_outer_refit_deltas.parquet</t>
+          <t>outputs/local/D5_reference_window_library.xlsx</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>7921</v>
+        <v>228952</v>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>1601955bc59dfd0da87cd33e695f16ac974ad0be8ecacbdb23dfe465599ce7bf</t>
+          <t>12bb084003accca5fd0e85f42191286a56a27c7016b617296cde45ff4004edf1</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>outputs/publication/D5_outer_refit_summary.parquet</t>
+          <t>outputs/local/D5_regime_state.parquet</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>6681</v>
+        <v>3658910</v>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>9ea7de7e9e34e2bc3b5c657dd72bded594918e0310ad7e231a2610ef45253f30</t>
+          <t>622dd0f5ed1473ae5de464e4207e51ff9470de209cadcee9b30cbac92f9392e8</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>outputs/publication/D5_publication_audit_manifest.json</t>
+          <t>outputs/local/D5_regime_state.xlsx</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>14709</v>
+        <v>45834835</v>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>39ebf4d77c3e9e04c9a622a204f137ec2789aa8e9fed6d7ba857138eb0feb16b</t>
+          <t>427fe81df8b7861210e267f694058376a754fa724e0bbafe1b07208e32787485</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>outputs/publication/D5_publication_audit_tables.xlsx</t>
+          <t>outputs/local/D5_report_interface.parquet</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>31653</v>
+        <v>1171194</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>d60260e90fd48ffe9f5eb643639d0b94f863e9346dc922ec16b33499578dc930</t>
+          <t>f057e0a8037282fb43a71a94d7043c7bd3de2b4c8fa9865365bcf0427195dbda</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>outputs/publication/D5_PUBLICATION_READINESS_AUDIT_v1.2.md</t>
+          <t>outputs/local/D5_report_interface.schema.json</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>7623</v>
+        <v>853</v>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>17e87ac6ee94ae2295677edb510245c808ce812f503bf29c4995e47e5b95b924</t>
+          <t>c740ff5a12c99a1a761c5f2ab45d12f5174aaac3b2201e58e6d67a1a8c87c06e</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>outputs/publication/D5_risk_coverage.parquet</t>
+          <t>outputs/local/D5_report_interface.xlsx</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>5064</v>
+        <v>11410677</v>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>eb0caf68ddfdc8203a64254c3aa277304432bb3fa762cb19e0b9123740a49508</t>
+          <t>f9040450b3fb8204f2fea44f92c003d1cdc2acf900a29715ee732a8b9b450aae</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>outputs/publication/D5_support_sensitivity.parquet</t>
+          <t>outputs/local/D5_sensor_influence.parquet</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>5871</v>
+        <v>6011187</v>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>f6ee73f3893ed53682e63122e9220948cc97ffa0c9ead47b20b6b2c739de9fda</t>
+          <t>a9270494760fcb4ae501abcf54c50e813ca74d6306d7fbca94d7ef1a1d1730a2</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>outputs/publication/D5_target_influence.parquet</t>
+          <t>outputs/local/D5_sensor_influence.xlsx</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>8537</v>
+        <v>16403976</v>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>13af4a843ab3f1942fe634e88b6bb8badd884917e8a2533d602bff89b59f54ff</t>
+          <t>338920c1db9c7b1bc500fa43d92f02f6165187545a79f696771287bfd877a9a0</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>outputs/publication/FigD5_6_validation_coverage_source_data.xlsx</t>
+          <t>outputs/local/D5_sensor_profile_summary.xlsx</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>10606</v>
+        <v>7442</v>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>568846bf82c1a60ce496d7724149414ac469e6978464d9a284e5b7a4717ae6e0</t>
+          <t>aef38bd66378a9ae3b2c76a848f1ef4d51d504616c435440e45f99eadf9fb5a9</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>outputs/publication/FigD5_7_D4_D5_complementarity_source_data.xlsx</t>
+          <t>outputs/local/D5_spatial_evidence.parquet</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>11724</v>
+        <v>6146048</v>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>6838f382cacb25c9f1c1eff8afaebee4dccb71642e079232bed30438496ca8ca</t>
+          <t>4edb2bd1af0cbdac8fc61382508099137349f67f6ce70da4ee1831848bfe3733</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>outputs/publication/FigD5_8_dimension_availability_sensitivity_source_data.xlsx</t>
+          <t>outputs/local/D5_spatial_evidence.xlsx</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>6490</v>
+        <v>15958642</v>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>1ace1bc7ebbe577865e112f1ffb4910fc9a384bcfe46e8ab2d1ff0beb8e5f746</t>
+          <t>6e2a433bcdb115b841f269c5eb5184623502c7221234da51b8ade0377c120327</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>outputs/publication/FigD5_9_target_support_robustness_source_data.xlsx</t>
+          <t>outputs/local/D5_spatial_templates.template_bundle.json</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>7501</v>
+        <v>542571</v>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>43dc129f8d845916e79369d3dd5c07546c375da8a8b64127945fa9c6f2f9bd8d</t>
+          <t>704238fcb5551593e569bdb3e015f04cb710815fdeccbb8aa28ba9a0c7e59ace</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_CURRENT_RELEASE.md</t>
+          <t>outputs/local/D5_spatial_templates.xlsx</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>1058</v>
+        <v>190694</v>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>53e0d073ef332fc162b7db37c204f7e803ab19e193a8adce3354f8cb59ac06aa</t>
+          <t>6fc3291e19dd0663ccd33db897edbf39e67f54e7db7b1fa8de0648d06d82c6bc</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_EXPERT_REPORT_v2.1.docx</t>
+          <t>outputs/local/D5_support_assessment.parquet</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>2047657</v>
+        <v>52815</v>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>8e5db363b70bd05b8584eb191b764d1d2beee31c2be738b56f44c9902c67fb04</t>
+          <t>00d3ed69dc3899db48c841bb56c6664bc1832e365fd5fa5c13130b6d231e5750</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_EXPERT_REPORT_v2.1.md</t>
+          <t>outputs/local/D5_support_assessment.xlsx</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>7814</v>
+        <v>28036</v>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>6de0e55c9c7f57f2c030d48076b3da316a94d53167e1c1e9d164031972691657</t>
+          <t>34df65d8e4329d166c69a9bc505bb97a8397e537f323c5be392fba093827dd98</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_EXPERT_REPORT_v2.2.docx</t>
+          <t>outputs/local/D5_topology_drift_alerts.parquet</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>2107226</v>
+        <v>10824</v>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>9dfbe96a145765a0e22e8452ec1a76f759ae52cd201b71694aa7c7e815fd8d8b</t>
+          <t>59d05a6c138fc18e295611bb0e39f469c07f6a25522ed809ea4f76ca018a908a</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_EXPERT_REPORT_v2.2.md</t>
+          <t>outputs/local/D5_topology_drift_alerts.xlsx</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>8480</v>
+        <v>9965</v>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>5f9333b22a9d8dc1b40d9ac2f1f684ee851785bf1f742be406e6433cfc841cfd</t>
+          <t>7262caaddcf1713a512e6dd52157f3f0e4bee9ae2642dcaf63eed60ff9ce9a87</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_EXPERT_REPORT_v2.3.docx</t>
+          <t>outputs/local/D5_topology_evidence.yaml</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>2056532</v>
+        <v>2342</v>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>19b15492f9b09b02820cf4ff0effd41c672a7dd0a99a42eef3886c732b622fe5</t>
+          <t>50abd276a9e6bbf26acb9a22d3a796ca63423d363a036422dc57c6bdfeb71920</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_EXPERT_REPORT_v2.3.md</t>
+          <t>outputs/local/D5_topology_registry.json</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>9043</v>
+        <v>14821</v>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>93baa7ffe8d1d92abac60ce6896dd742d71410bb89c771ab5d8e73c9bc3d6b57</t>
+          <t>6efbf6722e2caecabf2d9999637d48bbb7c4d630dc3e9354982ed89d750965bc</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_EXPERT_REPORT_v2.4.docx</t>
+          <t>outputs/local/D5_topology_registry.schema.json</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>3942265</v>
+        <v>1301</v>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>be2dedbef7c560882c3cb5a89778b001e9428c2003f987ed1dfb20dd1a9da3b4</t>
+          <t>0f4c6e9e6d510996d1435efd1810b4a1eaca35a989b7f3d78187e29f8ce9584e</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_EXPERT_REPORT_v2.4.md</t>
+          <t>outputs/local/D5_topology_registry.xlsx</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>10364</v>
+        <v>11679</v>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>159d6a0c126fa64bc59844f3deeb4494baab692d9a7d559f35cfa6ba94957c80</t>
+          <t>7aa5db4087c2346acc99d827f7c3a0bd49ce90540fb2ec8f56664c82b14e36ff</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_FIGURE_CAPTIONS_v2.1.md</t>
+          <t>outputs/local/D5_topology_registry.yaml</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>2282</v>
+        <v>2838</v>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>dd5ca9eea1365f682a5166e6f8e11da3da1b6ce06652795ba6bd0112a5711bc0</t>
+          <t>46e191549a0c768ee947bff4d98f26f38a93ecbce380ab4ff8114d2885dd29f9</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_FIGURE_CAPTIONS_v2.2.md</t>
+          <t>outputs/local/D5_validation_results.xlsx</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>2185</v>
+        <v>64326</v>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>4e3e50df15c243b7c789337fb51e9fe8f350c3815f05b408b6dd2f8aad9c4067</t>
+          <t>b4a0f5586b1108b945dba84b87a47a7f387c11fa182de0c506977f3c9870efff</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_FIGURE_CAPTIONS_v2.3.md</t>
+          <t>outputs/local/D5_zone_consensus.parquet</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>2471</v>
+        <v>1618880</v>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>5aace3b407bf260ee6a54a95a25736b01d1ec2831a95823a45288d40270b532c</t>
+          <t>0cb43651f4dc8c4a7f378cfe3be964a688e7df7a2ff45052f649259b415cdb8c</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_FIGURE_CAPTIONS_v2.4.md</t>
+          <t>outputs/local/D5_zone_consensus.xlsx</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>4538</v>
+        <v>7277838</v>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>3bab49b975e41041916bbf003bedcaf390c7752a5418272d83e265867375eafc</t>
+          <t>f43c5554c5a0c9f3e50e38f51bc0db270a9c819c3a00a9f3dc23ae658b7e7149</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_PROJECT_DIRECTORY_GUIDE_v2.1.docx</t>
+          <t>outputs/plot_data/D5_plot_data.csv</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>40336</v>
+        <v>19888935</v>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>c2da3e9cca5ef0a5e83b63089e8deeb7299a7e0e7735c0b4751cd47f2fc47844</t>
+          <t>2f64df8e3b0855664a65c9cbd2245e71fc82ffd28583668cf16f623c7fff91b4</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_PROJECT_DIRECTORY_GUIDE_v2.1.md</t>
+          <t>outputs/plot_data/D5_plot_data.parquet</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>5333</v>
+        <v>711420</v>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>0303a5bbdc16689493eb5b3826d95bf7c23fc4405284ef7db01d13b5a1d1b045</t>
+          <t>9b5ba34ed66d3bf3466d541b2d6474860157c8905a1ae15e3cba3bc33cd2b5ad</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_PROJECT_DIRECTORY_GUIDE_v2.2.docx</t>
+          <t>outputs/plot_data/D5_plot_data_manifest.json</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>40363</v>
+        <v>519</v>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>eada32c51f435a6355dc873b748b4f894cbbc17bedfc4be6090371aa323aea5e</t>
+          <t>abcf4000817bd11e46428d772225579a90b6f3584bff3de23ae7c760d36c0e7e</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_PROJECT_DIRECTORY_GUIDE_v2.2.md</t>
+          <t>outputs/publication/D5_coverage_strata.parquet</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>5307</v>
+        <v>5837</v>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>b63d3b48b8902ad31fcbeac70f218c2c3abd2b1ee4293aff45cbc89fe16b950b</t>
+          <t>f4da589996c29b4e710131be262c3efdaa0fb822e051293f1310365aaf0e7b75</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_PROJECT_DIRECTORY_GUIDE_v2.3.docx</t>
+          <t>outputs/publication/D5_coverage_summary.parquet</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>40364</v>
+        <v>2879</v>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>788d71134331e7d994e157cbfb511ef1f5966eb546d05ea3a77a8b2dd90c2fce</t>
+          <t>54201e6be7009f8ed97eb53e8abd9d8d33766757486839e1d1650d09bf1718c6</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_PROJECT_DIRECTORY_GUIDE_v2.3.md</t>
+          <t>outputs/publication/D5_d4_d5_composite.parquet</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>5459</v>
+        <v>6628</v>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>0308ed8c677cbbb3581e4022bbc99623af3de79cf83fc9283b160fd54cb8d503</t>
+          <t>f6245e6b95476622c5ccdbabdd9819e0c5c449e8e2f38797f396dba21861150d</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_PROJECT_DIRECTORY_GUIDE_v2.4.docx</t>
+          <t>outputs/publication/D5_d4_d5_dependence.parquet</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>40394</v>
+        <v>8012</v>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>1072270e8cf7d3efdddc267aa49b1cd19f52b934979bb7b55636ac06fd50eec8</t>
+          <t>cc38200304298af4af8178ed2d35226ea9f75fb5608608fc83a1ee472b8d718b</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>outputs/reports/D5_PROJECT_DIRECTORY_GUIDE_v2.4.md</t>
+          <t>outputs/publication/D5_d4_d5_joint_sample.parquet</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>5736</v>
+        <v>302250</v>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>c1f9a23a8393c682257095dfa31c53a07256a104a52ccf89d1b83140d1246590</t>
+          <t>62daa89703d04a89b478c644f0eaa52343b8f2911f7ab56cb0f061e8614270c6</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>outputs/reports/nature_figure_bundle_audit.json</t>
+          <t>outputs/publication/D5_d4_d5_low_tail_overlap.parquet</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>2409</v>
+        <v>6549</v>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>da3ebd141c082e91a1745abc60394a9bc5c09de0cd31ad6297aa5cafc4d49756</t>
+          <t>feb6a3dccb134f99fdb07ddc02fd5fa8e1a415c5c0a6d0ea5c60d693409212bb</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>outputs/sensitivity/D5_sensitivity_manifest.json</t>
+          <t>outputs/publication/D5_d4_d5_stratified_rho.parquet</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>2345</v>
+        <v>12046</v>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>71ddb925f1c43c2bb363be78cb221f6a90ed9d1bce2beb713989957efcb0b8d8</t>
+          <t>b551d102dd73641908975d207793d15f892655b9ce719faba40f8c390cfcd961</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>outputs/sensitivity/D5_shadow_scores.parquet</t>
+          <t>outputs/publication/D5_decision_register.parquet</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>2987712</v>
+        <v>4954</v>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>a54b95d4cada7ab1f9a1e4bd7723d29f46c9e3c19de2bcab6f52a9da161ba5fc</t>
+          <t>2c82c18cd5897448165a93ce87e3423feccbe35155e74cee4d89cb6c7ad667dc</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>outputs/sensitivity/D5_shadow_scores.xlsx</t>
+          <t>outputs/publication/D5_dimension_availability.parquet</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>10004039</v>
+        <v>12550</v>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>1229f93be5258226bfbdc36daab2ceb3aa2b475485c1fa0392cc15ec148a97f9</t>
+          <t>f34750499b681fb5eefe3f811fbbec3a4d0570f45ca71a850a191b4a67c93680</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>outputs/sensitivity/D5_shadow_template_shift.xlsx</t>
+          <t>outputs/publication/D5_localization.parquet</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>41680</v>
+        <v>6980</v>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>3f68e2e6f4d6bc46aa021613f6b8ee25bb562d0798f1896ef47555b36c89fe35</t>
+          <t>e63682e2c8a0ebeb772d9d0eae21b4be654b370f853eb939376249c595ddfcff</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>outputs/sensitivity/D5_track_invariance.xlsx</t>
+          <t>outputs/publication/D5_monthly_coverage.parquet</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>14538</v>
+        <v>6986</v>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>c9ed72b9a91d1fa854692c1cabf77687a652bf9723a7d405b4fbc08cf5b6c1c0</t>
+          <t>ecf86809c3c74c92e8c173d9f21652b60a02212bd7dcee24b6f44b815fe639fc</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>outputs/shadow_v2/D5_graph_structure_learning_shadow.parquet</t>
+          <t>outputs/publication/D5_outer_refit_deltas.parquet</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>9388</v>
+        <v>7921</v>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>f65546587bfb8c5a13efa5af7a38f57820bb3467cbd974c3bfad3c369a88f2c7</t>
+          <t>1601955bc59dfd0da87cd33e695f16ac974ad0be8ecacbdb23dfe465599ce7bf</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>outputs/shadow_v2/D5_graph_structure_learning_shadow.xlsx</t>
+          <t>outputs/publication/D5_outer_refit_summary.parquet</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>8325</v>
+        <v>6681</v>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>b5a4109a1f1e707a2bc54497df9a808bd01cf23a9094aed4a77ff885fef49653</t>
+          <t>9ea7de7e9e34e2bc3b5c657dd72bded594918e0310ad7e231a2610ef45253f30</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
+          <t>outputs/publication/D5_publication_audit_manifest.json</t>
+        </is>
+      </c>
+      <c r="B135" t="n">
+        <v>15638</v>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>ec401c6052d3c339e95f508a24baf4b7c5f74f499518bf71e2faebf27c0f79e7</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>outputs/publication/D5_publication_audit_tables.xlsx</t>
+        </is>
+      </c>
+      <c r="B136" t="n">
+        <v>1642024</v>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>8a654d3b301ba058725d5dfe490ecdc38435b413d1f72d41e88a4caeb81e8521</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>outputs/publication/D5_PUBLICATION_READINESS_AUDIT_v1.2.md</t>
+        </is>
+      </c>
+      <c r="B137" t="n">
+        <v>7623</v>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>17e87ac6ee94ae2295677edb510245c808ce812f503bf29c4995e47e5b95b924</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>outputs/publication/D5_risk_coverage.parquet</t>
+        </is>
+      </c>
+      <c r="B138" t="n">
+        <v>8219</v>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>c3293962b24ffdb787294c67a482f570bd2ea9610bd0bf2c864812ac0580d7ba</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>outputs/publication/D5_support_sensitivity.parquet</t>
+        </is>
+      </c>
+      <c r="B139" t="n">
+        <v>5871</v>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>f6ee73f3893ed53682e63122e9220948cc97ffa0c9ead47b20b6b2c739de9fda</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>outputs/publication/D5_target_influence.parquet</t>
+        </is>
+      </c>
+      <c r="B140" t="n">
+        <v>8537</v>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>13af4a843ab3f1942fe634e88b6bb8badd884917e8a2533d602bff89b59f54ff</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>outputs/publication/FigD5_6_validation_coverage_source_data.xlsx</t>
+        </is>
+      </c>
+      <c r="B141" t="n">
+        <v>11472</v>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>2635ef66dc17d868bae2c37be718667dca0096d410d71ed5f788dc7af663e24b</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>outputs/publication/FigD5_7_D4_D5_complementarity_source_data.xlsx</t>
+        </is>
+      </c>
+      <c r="B142" t="n">
+        <v>1621841</v>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>47c67a4b9f0c44e6035357109f900ff3c36492ce2eadb5c63bacfc12ce613877</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>outputs/publication/FigD5_8_dimension_availability_sensitivity_source_data.xlsx</t>
+        </is>
+      </c>
+      <c r="B143" t="n">
+        <v>6490</v>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>40461b5d043772a94853ea31193129a848492916623be61b848fb96fad0219e9</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>outputs/publication/FigD5_9_target_support_robustness_source_data.xlsx</t>
+        </is>
+      </c>
+      <c r="B144" t="n">
+        <v>7501</v>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>8919815720a6ad0517db7875398c0c6dfcc2e712e4637404d626236730cd66c3</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>outputs/reports/D5_CURRENT_RELEASE.md</t>
+        </is>
+      </c>
+      <c r="B145" t="n">
+        <v>1058</v>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>720b831533e86a9c3206a20a75f825a28700075c85f488fce074ec8e5c1cad3d</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>outputs/reports/D5_EXPERT_REPORT_v2.1.docx</t>
+        </is>
+      </c>
+      <c r="B146" t="n">
+        <v>2047657</v>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>8e5db363b70bd05b8584eb191b764d1d2beee31c2be738b56f44c9902c67fb04</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>outputs/reports/D5_EXPERT_REPORT_v2.1.md</t>
+        </is>
+      </c>
+      <c r="B147" t="n">
+        <v>7814</v>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>6de0e55c9c7f57f2c030d48076b3da316a94d53167e1c1e9d164031972691657</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>outputs/reports/D5_EXPERT_REPORT_v2.2.docx</t>
+        </is>
+      </c>
+      <c r="B148" t="n">
+        <v>2107226</v>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>9dfbe96a145765a0e22e8452ec1a76f759ae52cd201b71694aa7c7e815fd8d8b</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>outputs/reports/D5_EXPERT_REPORT_v2.2.md</t>
+        </is>
+      </c>
+      <c r="B149" t="n">
+        <v>8480</v>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>5f9333b22a9d8dc1b40d9ac2f1f684ee851785bf1f742be406e6433cfc841cfd</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>outputs/reports/D5_EXPERT_REPORT_v2.3.docx</t>
+        </is>
+      </c>
+      <c r="B150" t="n">
+        <v>2056532</v>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>19b15492f9b09b02820cf4ff0effd41c672a7dd0a99a42eef3886c732b622fe5</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>outputs/reports/D5_EXPERT_REPORT_v2.3.md</t>
+        </is>
+      </c>
+      <c r="B151" t="n">
+        <v>9043</v>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>93baa7ffe8d1d92abac60ce6896dd742d71410bb89c771ab5d8e73c9bc3d6b57</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>outputs/reports/D5_EXPERT_REPORT_v2.4.docx</t>
+        </is>
+      </c>
+      <c r="B152" t="n">
+        <v>4646979</v>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>76018262af21c96aa3043999b8c1a5af9a3204af84ae3866bdbaa54cbb570765</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>outputs/reports/D5_EXPERT_REPORT_v2.4.md</t>
+        </is>
+      </c>
+      <c r="B153" t="n">
+        <v>13170</v>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>3f756be6fc359c29ce43b624a10149f8044b0f6db56e7b31579ab838eeed3225</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>outputs/reports/D5_FIGURE_CAPTIONS_v2.1.md</t>
+        </is>
+      </c>
+      <c r="B154" t="n">
+        <v>2282</v>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>dd5ca9eea1365f682a5166e6f8e11da3da1b6ce06652795ba6bd0112a5711bc0</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>outputs/reports/D5_FIGURE_CAPTIONS_v2.2.md</t>
+        </is>
+      </c>
+      <c r="B155" t="n">
+        <v>2185</v>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>4e3e50df15c243b7c789337fb51e9fe8f350c3815f05b408b6dd2f8aad9c4067</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>outputs/reports/D5_FIGURE_CAPTIONS_v2.3.md</t>
+        </is>
+      </c>
+      <c r="B156" t="n">
+        <v>2471</v>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>5aace3b407bf260ee6a54a95a25736b01d1ec2831a95823a45288d40270b532c</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>outputs/reports/D5_FIGURE_CAPTIONS_v2.4.md</t>
+        </is>
+      </c>
+      <c r="B157" t="n">
+        <v>7540</v>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>bcd441c228bc9e1405610080b04e3b0bbae743630249f964595d99b65abd4c73</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>outputs/reports/D5_PROJECT_DIRECTORY_GUIDE_v2.1.docx</t>
+        </is>
+      </c>
+      <c r="B158" t="n">
+        <v>40336</v>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>c2da3e9cca5ef0a5e83b63089e8deeb7299a7e0e7735c0b4751cd47f2fc47844</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>outputs/reports/D5_PROJECT_DIRECTORY_GUIDE_v2.1.md</t>
+        </is>
+      </c>
+      <c r="B159" t="n">
+        <v>5333</v>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>0303a5bbdc16689493eb5b3826d95bf7c23fc4405284ef7db01d13b5a1d1b045</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>outputs/reports/D5_PROJECT_DIRECTORY_GUIDE_v2.2.docx</t>
+        </is>
+      </c>
+      <c r="B160" t="n">
+        <v>40363</v>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>eada32c51f435a6355dc873b748b4f894cbbc17bedfc4be6090371aa323aea5e</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>outputs/reports/D5_PROJECT_DIRECTORY_GUIDE_v2.2.md</t>
+        </is>
+      </c>
+      <c r="B161" t="n">
+        <v>5307</v>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>b63d3b48b8902ad31fcbeac70f218c2c3abd2b1ee4293aff45cbc89fe16b950b</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>outputs/reports/D5_PROJECT_DIRECTORY_GUIDE_v2.3.docx</t>
+        </is>
+      </c>
+      <c r="B162" t="n">
+        <v>40364</v>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>788d71134331e7d994e157cbfb511ef1f5966eb546d05ea3a77a8b2dd90c2fce</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>outputs/reports/D5_PROJECT_DIRECTORY_GUIDE_v2.3.md</t>
+        </is>
+      </c>
+      <c r="B163" t="n">
+        <v>5459</v>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>0308ed8c677cbbb3581e4022bbc99623af3de79cf83fc9283b160fd54cb8d503</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>outputs/reports/D5_PROJECT_DIRECTORY_GUIDE_v2.4.docx</t>
+        </is>
+      </c>
+      <c r="B164" t="n">
+        <v>40394</v>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>f57e684efde41bd2ef99902ff89cd2ee20b9d927a48189303a0ac0887fb3712f</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>outputs/reports/D5_PROJECT_DIRECTORY_GUIDE_v2.4.md</t>
+        </is>
+      </c>
+      <c r="B165" t="n">
+        <v>7876</v>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>83b919cdef957f2b5ec1e9625343990e1c99d971b0ffdd7bdf246df9c062f2e9</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>outputs/reports/nature_figure_bundle_audit.json</t>
+        </is>
+      </c>
+      <c r="B166" t="n">
+        <v>7580</v>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>1d0c4e815827302ce0f19cc80dea5ff1028c03f19cf67f5676ad21c41e8290f3</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>outputs/sensitivity/D5_sensitivity_manifest.json</t>
+        </is>
+      </c>
+      <c r="B167" t="n">
+        <v>2345</v>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>71ddb925f1c43c2bb363be78cb221f6a90ed9d1bce2beb713989957efcb0b8d8</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>outputs/sensitivity/D5_shadow_scores.parquet</t>
+        </is>
+      </c>
+      <c r="B168" t="n">
+        <v>2987712</v>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>a54b95d4cada7ab1f9a1e4bd7723d29f46c9e3c19de2bcab6f52a9da161ba5fc</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>outputs/sensitivity/D5_shadow_scores.xlsx</t>
+        </is>
+      </c>
+      <c r="B169" t="n">
+        <v>10004039</v>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>1229f93be5258226bfbdc36daab2ceb3aa2b475485c1fa0392cc15ec148a97f9</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>outputs/sensitivity/D5_shadow_template_shift.xlsx</t>
+        </is>
+      </c>
+      <c r="B170" t="n">
+        <v>41680</v>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>3f68e2e6f4d6bc46aa021613f6b8ee25bb562d0798f1896ef47555b36c89fe35</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>outputs/sensitivity/D5_track_invariance.xlsx</t>
+        </is>
+      </c>
+      <c r="B171" t="n">
+        <v>14538</v>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>c9ed72b9a91d1fa854692c1cabf77687a652bf9723a7d405b4fbc08cf5b6c1c0</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>outputs/shadow_v2/D5_graph_structure_learning_shadow.parquet</t>
+        </is>
+      </c>
+      <c r="B172" t="n">
+        <v>9388</v>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>f65546587bfb8c5a13efa5af7a38f57820bb3467cbd974c3bfad3c369a88f2c7</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>outputs/shadow_v2/D5_graph_structure_learning_shadow.xlsx</t>
+        </is>
+      </c>
+      <c r="B173" t="n">
+        <v>8325</v>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>b5a4109a1f1e707a2bc54497df9a808bd01cf23a9094aed4a77ff885fef49653</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
           <t>outputs/shadow_v2/D5_shadow_v2_manifest.json</t>
         </is>
       </c>
-      <c r="B135" t="n">
+      <c r="B174" t="n">
         <v>263</v>
       </c>
-      <c r="C135" t="inlineStr">
+      <c r="C174" t="inlineStr">
         <is>
           <t>b031365e134ba1bfee32dd92c04e35cdff1e904f78937c214e008540551a11f3</t>
         </is>

</xml_diff>